<commit_message>
test case id renaming
</commit_message>
<xml_diff>
--- a/docs/test-cases.xlsx
+++ b/docs/test-cases.xlsx
@@ -672,7 +672,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Storefront (www.musticker.com/kr) + Admin panel (admin-panel.musticker.com) | Playwright + TypeScript | Workbook v1.1 | 2026-10-14</t>
+          <t>Storefront (www.musticker.com/kr) + Admin panel (admin-panel.musticker.com) | Playwright + TypeScript | Workbook v1.2 | 2026-10-14</t>
         </is>
       </c>
     </row>
@@ -824,7 +824,7 @@
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>Filter the Test Cases tab by Area, Priority, App or Automation. Only the orange-headed columns (Result, Defect ID, Tester, Executed On, Tester Notes) are for you to fill in.</t>
+          <t>Filter the Test Cases tab by Area, Priority, App or Automation. Only the orange-headed columns (Result, Defect ID, Tester, Executed On, Tester Notes) are for you to fill in. The Legacy ID column (Y) shows the ID a case had before workbook v1.2 (MS-V2-### / MS-ADM-###); it is for reference only.</t>
         </is>
       </c>
     </row>
@@ -968,7 +968,7 @@
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>Automated order placement on static-1 (dev-static-1): its checkout shows a Cloudflare bot check before payment that rejects automated browsers. MS-ADM-001 starts from a pre-placed seed order until the dev team exempts test traffic.</t>
+          <t>Automated order placement on static-1 (dev-static-1): its checkout shows a Cloudflare bot check before payment that rejects automated browsers. MS-ADMO-001 starts from a pre-placed seed order until the dev team exempts test traffic.</t>
         </is>
       </c>
     </row>
@@ -1169,7 +1169,7 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>Automated order placement on static-1 (Cloudflare check before payment). Admin cases in CI: the verification code needs a person - dev-static-1 has a tester OTP endpoint that could remove this (see MS-ADM-002), not used by the suite yet.</t>
+          <t>Automated order placement on static-1 (Cloudflare check before payment). Admin cases in CI: the verification code needs a person - dev-static-1 has a tester OTP endpoint that could remove this (see MS-ADMA-001), not used by the suite yet.</t>
         </is>
       </c>
     </row>
@@ -2410,7 +2410,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X176"/>
+  <dimension ref="A1:Y176"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -2434,6 +2434,7 @@
     <col width="12" customWidth="1" min="21" max="22"/>
     <col width="13" customWidth="1" min="23" max="23"/>
     <col width="28" customWidth="1" min="24" max="24"/>
+    <col width="14" customWidth="1" min="25" max="25"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -2557,11 +2558,16 @@
           <t>Tester Notes</t>
         </is>
       </c>
+      <c r="Y1" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Legacy ID</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="150" customHeight="1">
       <c r="A2" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-001</t>
+          <t>MS-NAV-001</t>
         </is>
       </c>
       <c r="B2" s="25" t="inlineStr">
@@ -2641,7 +2647,7 @@
       </c>
       <c r="P2" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-001 homepage loads with critical public content</t>
+          <t>MS-NAV-001 homepage loads with critical public content</t>
         </is>
       </c>
       <c r="Q2" s="25" t="inlineStr">
@@ -2666,11 +2672,16 @@
       <c r="V2" s="15" t="n"/>
       <c r="W2" s="15" t="n"/>
       <c r="X2" s="15" t="n"/>
+      <c r="Y2" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-001</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="150" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-002</t>
+          <t>MS-NAV-002</t>
         </is>
       </c>
       <c r="B3" s="25" t="inlineStr">
@@ -2749,7 +2760,7 @@
       </c>
       <c r="P3" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-002 header navigation opens each category product menu</t>
+          <t>MS-NAV-002 header navigation opens each category product menu</t>
         </is>
       </c>
       <c r="Q3" s="25" t="inlineStr">
@@ -2774,11 +2785,16 @@
       <c r="V3" s="15" t="n"/>
       <c r="W3" s="15" t="n"/>
       <c r="X3" s="15" t="n"/>
+      <c r="Y3" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-002</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="150" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-003</t>
+          <t>MS-NAV-003</t>
         </is>
       </c>
       <c r="B4" s="25" t="inlineStr">
@@ -2857,7 +2873,7 @@
       </c>
       <c r="P4" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-003 header search opens and finds hologram sticker content</t>
+          <t>MS-NAV-003 header search opens and finds hologram sticker content</t>
         </is>
       </c>
       <c r="Q4" s="25" t="inlineStr">
@@ -2882,11 +2898,16 @@
       <c r="V4" s="15" t="n"/>
       <c r="W4" s="15" t="n"/>
       <c r="X4" s="15" t="n"/>
+      <c r="Y4" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-003</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="150" customHeight="1">
       <c r="A5" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-004</t>
+          <t>MS-NAV-004</t>
         </is>
       </c>
       <c r="B5" s="25" t="inlineStr">
@@ -2964,7 +2985,7 @@
       </c>
       <c r="P5" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-004 empty cart opens without broken state</t>
+          <t>MS-NAV-004 empty cart opens without broken state</t>
         </is>
       </c>
       <c r="Q5" s="25" t="inlineStr">
@@ -2989,11 +3010,16 @@
       <c r="V5" s="15" t="n"/>
       <c r="W5" s="15" t="n"/>
       <c r="X5" s="15" t="n"/>
+      <c r="Y5" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-004</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="150" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-005</t>
+          <t>MS-NAV-005</t>
         </is>
       </c>
       <c r="B6" s="25" t="inlineStr">
@@ -3071,7 +3097,7 @@
       </c>
       <c r="P6" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-005 account icon routes anonymous users to authentication</t>
+          <t>MS-NAV-005 account icon routes anonymous users to authentication</t>
         </is>
       </c>
       <c r="Q6" s="25" t="inlineStr">
@@ -3096,11 +3122,16 @@
       <c r="V6" s="15" t="n"/>
       <c r="W6" s="15" t="n"/>
       <c r="X6" s="15" t="n"/>
+      <c r="Y6" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-005</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="150" customHeight="1">
       <c r="A7" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-020</t>
+          <t>MS-NAV-006</t>
         </is>
       </c>
       <c r="B7" s="25" t="inlineStr">
@@ -3178,7 +3209,7 @@
       </c>
       <c r="P7" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-020 footer legal and support links are reachable</t>
+          <t>MS-NAV-006 footer legal and support links are reachable</t>
         </is>
       </c>
       <c r="Q7" s="25" t="inlineStr">
@@ -3203,11 +3234,16 @@
       <c r="V7" s="15" t="n"/>
       <c r="W7" s="15" t="n"/>
       <c r="X7" s="15" t="n"/>
+      <c r="Y7" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-020</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="150" customHeight="1">
       <c r="A8" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-021</t>
+          <t>MS-NAV-007</t>
         </is>
       </c>
       <c r="B8" s="25" t="inlineStr">
@@ -3285,7 +3321,7 @@
       </c>
       <c r="P8" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-021 Korean locale control is stable</t>
+          <t>MS-NAV-007 Korean locale control is stable</t>
         </is>
       </c>
       <c r="Q8" s="25" t="inlineStr">
@@ -3298,7 +3334,7 @@
       </c>
       <c r="S8" s="25" t="inlineStr">
         <is>
-          <t>Conditional pass: with no KR button the test still passes on header visibility. It does not check that a locale menu opens or that Korean stays selected. Tags differ from test-case.md (@regression there, @smoke in code). The KR .locale-toggle button is a known color-contrast defect (see MS-V2-106).</t>
+          <t>Conditional pass: with no KR button the test still passes on header visibility. It does not check that a locale menu opens or that Korean stays selected. Tags differ from test-case.md (@regression there, @smoke in code). The KR .locale-toggle button is a known color-contrast defect (see MS-UX-004).</t>
         </is>
       </c>
       <c r="T8" s="14" t="inlineStr">
@@ -3310,11 +3346,16 @@
       <c r="V8" s="15" t="n"/>
       <c r="W8" s="15" t="n"/>
       <c r="X8" s="15" t="n"/>
+      <c r="Y8" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-021</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="150" customHeight="1">
       <c r="A9" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-022</t>
+          <t>MS-NAV-008</t>
         </is>
       </c>
       <c r="B9" s="25" t="inlineStr">
@@ -3395,7 +3436,7 @@
       </c>
       <c r="P9" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-022 home, search, cart, product config, and inquiry work on mobile</t>
+          <t>MS-NAV-008 home, search, cart, product config, and inquiry work on mobile</t>
         </is>
       </c>
       <c r="Q9" s="25" t="inlineStr">
@@ -3420,11 +3461,16 @@
       <c r="V9" s="15" t="n"/>
       <c r="W9" s="15" t="n"/>
       <c r="X9" s="15" t="n"/>
+      <c r="Y9" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-022</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="150" customHeight="1">
       <c r="A10" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-006</t>
+          <t>MS-DSC-001</t>
         </is>
       </c>
       <c r="B10" s="25" t="inlineStr">
@@ -3503,7 +3549,7 @@
       </c>
       <c r="P10" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-006 sticker category lists expected product links</t>
+          <t>MS-DSC-001 sticker category lists expected product links</t>
         </is>
       </c>
       <c r="Q10" s="25" t="inlineStr">
@@ -3528,11 +3574,16 @@
       <c r="V10" s="15" t="n"/>
       <c r="W10" s="15" t="n"/>
       <c r="X10" s="15" t="n"/>
+      <c r="Y10" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-006</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="150" customHeight="1">
       <c r="A11" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-007</t>
+          <t>MS-DSC-002</t>
         </is>
       </c>
       <c r="B11" s="25" t="inlineStr">
@@ -3611,7 +3662,7 @@
       </c>
       <c r="P11" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-007 roll sticker category lists expected product links</t>
+          <t>MS-DSC-002 roll sticker category lists expected product links</t>
         </is>
       </c>
       <c r="Q11" s="25" t="inlineStr">
@@ -3636,11 +3687,16 @@
       <c r="V11" s="15" t="n"/>
       <c r="W11" s="15" t="n"/>
       <c r="X11" s="15" t="n"/>
+      <c r="Y11" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-007</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="150" customHeight="1">
       <c r="A12" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-008</t>
+          <t>MS-DSC-003</t>
         </is>
       </c>
       <c r="B12" s="25" t="inlineStr">
@@ -3719,7 +3775,7 @@
       </c>
       <c r="P12" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-008 sheet sticker category lists expected product links</t>
+          <t>MS-DSC-003 sheet sticker category lists expected product links</t>
         </is>
       </c>
       <c r="Q12" s="25" t="inlineStr">
@@ -3744,11 +3800,16 @@
       <c r="V12" s="15" t="n"/>
       <c r="W12" s="15" t="n"/>
       <c r="X12" s="15" t="n"/>
+      <c r="Y12" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-008</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="150" customHeight="1">
       <c r="A13" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-015</t>
+          <t>MS-DSC-004</t>
         </is>
       </c>
       <c r="B13" s="25" t="inlineStr">
@@ -3827,7 +3888,7 @@
       </c>
       <c r="P13" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-015 FAQ topics and accordions are usable</t>
+          <t>MS-DSC-004 FAQ topics and accordions are usable</t>
         </is>
       </c>
       <c r="Q13" s="25" t="inlineStr">
@@ -3852,11 +3913,16 @@
       <c r="V13" s="15" t="n"/>
       <c r="W13" s="15" t="n"/>
       <c r="X13" s="15" t="n"/>
+      <c r="Y13" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-015</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="150" customHeight="1">
       <c r="A14" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-016</t>
+          <t>MS-DSC-005</t>
         </is>
       </c>
       <c r="B14" s="25" t="inlineStr">
@@ -3935,7 +4001,7 @@
       </c>
       <c r="P14" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-016 FAQ search filters and resets content</t>
+          <t>MS-DSC-005 FAQ search filters and resets content</t>
         </is>
       </c>
       <c r="Q14" s="25" t="inlineStr">
@@ -3960,11 +4026,16 @@
       <c r="V14" s="15" t="n"/>
       <c r="W14" s="15" t="n"/>
       <c r="X14" s="15" t="n"/>
+      <c r="Y14" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-016</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="150" customHeight="1">
       <c r="A15" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-039</t>
+          <t>MS-DSC-006</t>
         </is>
       </c>
       <c r="B15" s="25" t="inlineStr">
@@ -4043,7 +4114,7 @@
       </c>
       <c r="P15" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-039 about page loads hero, sub-nav, stats, and CTAs</t>
+          <t>MS-DSC-006 about page loads hero, sub-nav, stats, and CTAs</t>
         </is>
       </c>
       <c r="Q15" s="25" t="inlineStr">
@@ -4068,11 +4139,16 @@
       <c r="V15" s="15" t="n"/>
       <c r="W15" s="15" t="n"/>
       <c r="X15" s="15" t="n"/>
+      <c r="Y15" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-039</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="150" customHeight="1">
       <c r="A16" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-040</t>
+          <t>MS-DSC-007</t>
         </is>
       </c>
       <c r="B16" s="25" t="inlineStr">
@@ -4151,7 +4227,7 @@
       </c>
       <c r="P16" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-040 catalog page renders without error: ./stickers/sticker-sheet</t>
+          <t>MS-DSC-007 catalog page renders without error: ./stickers/sticker-sheet</t>
         </is>
       </c>
       <c r="Q16" s="25" t="inlineStr">
@@ -4176,11 +4252,16 @@
       <c r="V16" s="15" t="n"/>
       <c r="W16" s="15" t="n"/>
       <c r="X16" s="15" t="n"/>
+      <c r="Y16" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-040</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="150" customHeight="1">
       <c r="A17" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-009</t>
+          <t>MS-CFG-001</t>
         </is>
       </c>
       <c r="B17" s="25" t="inlineStr">
@@ -4260,7 +4341,7 @@
       </c>
       <c r="P17" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-009 die-cut sticker supports size and quantity selection</t>
+          <t>MS-CFG-001 die-cut sticker supports size and quantity selection</t>
         </is>
       </c>
       <c r="Q17" s="25" t="inlineStr">
@@ -4285,11 +4366,16 @@
       <c r="V17" s="15" t="n"/>
       <c r="W17" s="15" t="n"/>
       <c r="X17" s="15" t="n"/>
+      <c r="Y17" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-009</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="150" customHeight="1">
       <c r="A18" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-010</t>
+          <t>MS-CFG-002</t>
         </is>
       </c>
       <c r="B18" s="25" t="inlineStr">
@@ -4369,7 +4455,7 @@
       </c>
       <c r="P18" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-010 die-cut roll sticker supports size and quantity selection</t>
+          <t>MS-CFG-002 die-cut roll sticker supports size and quantity selection</t>
         </is>
       </c>
       <c r="Q18" s="25" t="inlineStr">
@@ -4382,7 +4468,7 @@
       </c>
       <c r="S18" s="25" t="inlineStr">
         <is>
-          <t>test-case.md mentions a per-unit price. The code only checks that some won amount is visible. The progression check is loose, as in MS-V2-009.</t>
+          <t>test-case.md mentions a per-unit price. The code only checks that some won amount is visible. The progression check is loose, as in MS-CFG-001.</t>
         </is>
       </c>
       <c r="T18" s="14" t="inlineStr">
@@ -4394,11 +4480,16 @@
       <c r="V18" s="15" t="n"/>
       <c r="W18" s="15" t="n"/>
       <c r="X18" s="15" t="n"/>
+      <c r="Y18" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-010</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="150" customHeight="1">
       <c r="A19" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-011</t>
+          <t>MS-CFG-003</t>
         </is>
       </c>
       <c r="B19" s="25" t="inlineStr">
@@ -4480,7 +4571,7 @@
       </c>
       <c r="P19" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-011 die-cut sheet sticker supports material, sheet size, and quantity selection</t>
+          <t>MS-CFG-003 die-cut sheet sticker supports material, sheet size, and quantity selection</t>
         </is>
       </c>
       <c r="Q19" s="25" t="inlineStr">
@@ -4505,11 +4596,16 @@
       <c r="V19" s="15" t="n"/>
       <c r="W19" s="15" t="n"/>
       <c r="X19" s="15" t="n"/>
+      <c r="Y19" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-011</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="150" customHeight="1">
       <c r="A20" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-012</t>
+          <t>MS-CFG-004</t>
         </is>
       </c>
       <c r="B20" s="25" t="inlineStr">
@@ -4589,7 +4685,7 @@
       </c>
       <c r="P20" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-012 custom size and quantity controls are reachable</t>
+          <t>MS-CFG-004 custom size and quantity controls are reachable</t>
         </is>
       </c>
       <c r="Q20" s="25" t="inlineStr">
@@ -4615,11 +4711,16 @@
       <c r="V20" s="15" t="n"/>
       <c r="W20" s="15" t="n"/>
       <c r="X20" s="15" t="n"/>
+      <c r="Y20" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-012</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="150" customHeight="1">
       <c r="A21" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-013</t>
+          <t>MS-CFG-005</t>
         </is>
       </c>
       <c r="B21" s="25" t="inlineStr">
@@ -4697,7 +4798,7 @@
       </c>
       <c r="P21" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-013 product trust and delivery promises are visible</t>
+          <t>MS-CFG-005 product trust and delivery promises are visible</t>
         </is>
       </c>
       <c r="Q21" s="25" t="inlineStr">
@@ -4722,11 +4823,16 @@
       <c r="V21" s="15" t="n"/>
       <c r="W21" s="15" t="n"/>
       <c r="X21" s="15" t="n"/>
+      <c r="Y21" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-013</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="150" customHeight="1">
       <c r="A22" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-014</t>
+          <t>MS-CFG-006</t>
         </is>
       </c>
       <c r="B22" s="25" t="inlineStr">
@@ -4805,7 +4911,7 @@
       </c>
       <c r="P22" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-014 product review carousel is usable</t>
+          <t>MS-CFG-006 product review carousel is usable</t>
         </is>
       </c>
       <c r="Q22" s="25" t="inlineStr">
@@ -4830,11 +4936,16 @@
       <c r="V22" s="15" t="n"/>
       <c r="W22" s="15" t="n"/>
       <c r="X22" s="15" t="n"/>
+      <c r="Y22" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-014</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="150" customHeight="1">
       <c r="A23" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-050</t>
+          <t>MS-CFG-007</t>
         </is>
       </c>
       <c r="B23" s="25" t="inlineStr">
@@ -4915,7 +5026,7 @@
       </c>
       <c r="P23" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-050 원형 판스티커 supports material, size, and quantity selection through to cart</t>
+          <t>MS-CFG-007 원형 판스티커 supports material, size, and quantity selection through to cart</t>
         </is>
       </c>
       <c r="Q23" s="25" t="inlineStr">
@@ -4940,11 +5051,16 @@
       <c r="V23" s="15" t="n"/>
       <c r="W23" s="15" t="n"/>
       <c r="X23" s="15" t="n"/>
+      <c r="Y23" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-050</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="150" customHeight="1">
       <c r="A24" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-051</t>
+          <t>MS-CFG-008</t>
         </is>
       </c>
       <c r="B24" s="25" t="inlineStr">
@@ -5023,7 +5139,7 @@
       </c>
       <c r="P24" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-051 circle sheet sticker: custom individual size recalculates the whole quantity price ladder</t>
+          <t>MS-CFG-008 circle sheet sticker: custom individual size recalculates the whole quantity price ladder</t>
         </is>
       </c>
       <c r="Q24" s="25" t="inlineStr">
@@ -5036,7 +5152,7 @@
       </c>
       <c r="S24" s="25" t="inlineStr">
         <is>
-          <t>The title and test-case.md say the whole price ladder is recalculated. The code only checks that a won amount is visible and 다음 단계 is enabled; it does not compare prices before and after. Field labels differ by environment: dev uses 가로/세로 placeholders, while production uses 너비/높이 captions with an "예: 30" placeholder. test-case.md says the helper retries the click once; it now retries up to 5 times. The fractional per-unit price (e.g. 8.582원) is accepted behavior, not a defect (MS-V2-059 withdrawn).</t>
+          <t>The title and test-case.md say the whole price ladder is recalculated. The code only checks that a won amount is visible and 다음 단계 is enabled; it does not compare prices before and after. Field labels differ by environment: dev uses 가로/세로 placeholders, while production uses 너비/높이 captions with an "예: 30" placeholder. test-case.md says the helper retries the click once; it now retries up to 5 times. The fractional per-unit price (e.g. 8.582원) is accepted behavior, not a defect (MS-CFG-016 withdrawn).</t>
         </is>
       </c>
       <c r="T24" s="14" t="inlineStr">
@@ -5048,11 +5164,16 @@
       <c r="V24" s="15" t="n"/>
       <c r="W24" s="15" t="n"/>
       <c r="X24" s="15" t="n"/>
+      <c r="Y24" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-051</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="150" customHeight="1">
       <c r="A25" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-052</t>
+          <t>MS-CFG-009</t>
         </is>
       </c>
       <c r="B25" s="25" t="inlineStr">
@@ -5129,7 +5250,7 @@
       </c>
       <c r="P25" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-052 circle sheet sticker: bulk quantity tiers surface a bigger discount than smaller tiers</t>
+          <t>MS-CFG-009 circle sheet sticker: bulk quantity tiers surface a bigger discount than smaller tiers</t>
         </is>
       </c>
       <c r="Q25" s="25" t="inlineStr">
@@ -5142,7 +5263,7 @@
       </c>
       <c r="S25" s="25" t="inlineStr">
         <is>
-          <t>Changed by 2026-10-14: sheet stickers now show a discount on every tier (10시트 reads -4% against a 6,900원 list price), so the old check that small tiers show no badge no longer holds. Badge values vary with the price table, so only their order is asserted. The die-cut and roll equivalents (MS-V2-064, MS-V2-065) still show no badge at 10개 and are unchanged.</t>
+          <t>Changed by 2026-10-14: sheet stickers now show a discount on every tier (10시트 reads -4% against a 6,900원 list price), so the old check that small tiers show no badge no longer holds. Badge values vary with the price table, so only their order is asserted. The die-cut and roll equivalents (MS-CFG-021, MS-CFG-022) still show no badge at 10개 and are unchanged.</t>
         </is>
       </c>
       <c r="T25" s="14" t="inlineStr">
@@ -5154,11 +5275,16 @@
       <c r="V25" s="15" t="n"/>
       <c r="W25" s="15" t="n"/>
       <c r="X25" s="15" t="n"/>
+      <c r="Y25" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-052</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="150" customHeight="1">
       <c r="A26" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-053</t>
+          <t>MS-CFG-010</t>
         </is>
       </c>
       <c r="B26" s="25" t="inlineStr">
@@ -5214,7 +5340,7 @@
       </c>
       <c r="K26" s="25" t="inlineStr">
         <is>
-          <t>the 어떻게 주문하시겠어요? chooser appears with the three ways to order (see MS-V2-050); after choosing the file, the dropzone shows "sample-design.png"; after 파일로 주문하기 the 장바구니 미리보기 (cart preview) drawer opens and contains a line item named "원형 판스티커" showing "수량: 10"; 장바구니 보기 leads to /kr/cart, where the 원형 판스티커 row shows either "이미지 추가" or "이미지 변경".</t>
+          <t>the 어떻게 주문하시겠어요? chooser appears with the three ways to order (see MS-CFG-007); after choosing the file, the dropzone shows "sample-design.png"; after 파일로 주문하기 the 장바구니 미리보기 (cart preview) drawer opens and contains a line item named "원형 판스티커" showing "수량: 10"; 장바구니 보기 leads to /kr/cart, where the 원형 판스티커 row shows either "이미지 추가" or "이미지 변경".</t>
         </is>
       </c>
       <c r="L26" s="13" t="inlineStr">
@@ -5239,7 +5365,7 @@
       </c>
       <c r="P26" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-053 circle sheet sticker: design upload modal accepts an order note and a design file before adding to cart</t>
+          <t>MS-CFG-010 circle sheet sticker: design upload modal accepts an order note and a design file before adding to cart</t>
         </is>
       </c>
       <c r="Q26" s="25" t="inlineStr">
@@ -5264,11 +5390,16 @@
       <c r="V26" s="15" t="n"/>
       <c r="W26" s="15" t="n"/>
       <c r="X26" s="15" t="n"/>
+      <c r="Y26" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-053</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="150" customHeight="1">
       <c r="A27" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-054</t>
+          <t>MS-CFG-011</t>
         </is>
       </c>
       <c r="B27" s="25" t="inlineStr">
@@ -5348,7 +5479,7 @@
       </c>
       <c r="P27" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-054 circle sheet sticker: editing material from the cart preview drawer recalculates the line price</t>
+          <t>MS-CFG-011 circle sheet sticker: editing material from the cart preview drawer recalculates the line price</t>
         </is>
       </c>
       <c r="Q27" s="25" t="inlineStr">
@@ -5373,11 +5504,16 @@
       <c r="V27" s="15" t="n"/>
       <c r="W27" s="15" t="n"/>
       <c r="X27" s="15" t="n"/>
+      <c r="Y27" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-054</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="150" customHeight="1">
       <c r="A28" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-055</t>
+          <t>MS-CFG-012</t>
         </is>
       </c>
       <c r="B28" s="25" t="inlineStr">
@@ -5456,7 +5592,7 @@
       </c>
       <c r="P28" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-055 circle sheet sticker: cart preview drawer "장바구니 보기" hands off to the full cart page with the item intact</t>
+          <t>MS-CFG-012 circle sheet sticker: cart preview drawer "장바구니 보기" hands off to the full cart page with the item intact</t>
         </is>
       </c>
       <c r="Q28" s="25" t="inlineStr">
@@ -5481,11 +5617,16 @@
       <c r="V28" s="15" t="n"/>
       <c r="W28" s="15" t="n"/>
       <c r="X28" s="15" t="n"/>
+      <c r="Y28" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-055</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="150" customHeight="1">
       <c r="A29" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-056</t>
+          <t>MS-CFG-013</t>
         </is>
       </c>
       <c r="B29" s="25" t="inlineStr">
@@ -5566,7 +5707,7 @@
       </c>
       <c r="P29" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-056 circle sheet sticker: full cart page "사이즈 변경" dialog exposes material + size only (no quantity), and updates price</t>
+          <t>MS-CFG-013 circle sheet sticker: full cart page "사이즈 변경" dialog exposes material + size only (no quantity), and updates price</t>
         </is>
       </c>
       <c r="Q29" s="25" t="inlineStr">
@@ -5579,7 +5720,7 @@
       </c>
       <c r="S29" s="25" t="inlineStr">
         <is>
-          <t>Having no quantity field in this dialog is intended, not a defect: quantity is edited only through the row select (MS-V2-057). test-case.md says the dialog shows 소재 and 개별 사이즈; the code does not check those labels, only that 수량 is absent. The default sheet material 무광 화이트 was labelled PVC 매트 until early October 2026. Uses 10시트, the smallest tier since early October 2026: 5시트 was dropped, and until the selector was fixed on 2026-10-14 asking for 5 silently picked 50시트.</t>
+          <t>Having no quantity field in this dialog is intended, not a defect: quantity is edited only through the row select (MS-CFG-014). test-case.md says the dialog shows 소재 and 개별 사이즈; the code does not check those labels, only that 수량 is absent. The default sheet material 무광 화이트 was labelled PVC 매트 until early October 2026. Uses 10시트, the smallest tier since early October 2026: 5시트 was dropped, and until the selector was fixed on 2026-10-14 asking for 5 silently picked 50시트.</t>
         </is>
       </c>
       <c r="T29" s="14" t="inlineStr">
@@ -5591,11 +5732,16 @@
       <c r="V29" s="15" t="n"/>
       <c r="W29" s="15" t="n"/>
       <c r="X29" s="15" t="n"/>
+      <c r="Y29" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-056</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="150" customHeight="1">
       <c r="A30" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-057</t>
+          <t>MS-CFG-014</t>
         </is>
       </c>
       <c r="B30" s="25" t="inlineStr">
@@ -5676,7 +5822,7 @@
       </c>
       <c r="P30" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-057 circle sheet sticker: full cart page row quantity select updates price without a separate confirm step</t>
+          <t>MS-CFG-014 circle sheet sticker: full cart page row quantity select updates price without a separate confirm step</t>
         </is>
       </c>
       <c r="Q30" s="25" t="inlineStr">
@@ -5701,11 +5847,16 @@
       <c r="V30" s="15" t="n"/>
       <c r="W30" s="15" t="n"/>
       <c r="X30" s="15" t="n"/>
+      <c r="Y30" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-057</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="150" customHeight="1">
       <c r="A31" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-058</t>
+          <t>MS-CFG-015</t>
         </is>
       </c>
       <c r="B31" s="25" t="inlineStr">
@@ -5782,7 +5933,7 @@
       </c>
       <c r="P31" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-058 원형 판스티커 size-guide illustrations have meaningful, localized alt text</t>
+          <t>MS-CFG-015 원형 판스티커 size-guide illustrations have meaningful, localized alt text</t>
         </is>
       </c>
       <c r="Q31" s="25" t="inlineStr">
@@ -5807,11 +5958,16 @@
       <c r="V31" s="15" t="n"/>
       <c r="W31" s="15" t="n"/>
       <c r="X31" s="15" t="n"/>
+      <c r="Y31" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-058</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="150" customHeight="1">
       <c r="A32" s="16" t="inlineStr">
         <is>
-          <t>MS-V2-059</t>
+          <t>MS-CFG-016</t>
         </is>
       </c>
       <c r="B32" s="25" t="inlineStr">
@@ -5911,11 +6067,16 @@
       <c r="V32" s="15" t="n"/>
       <c r="W32" s="15" t="n"/>
       <c r="X32" s="15" t="n"/>
+      <c r="Y32" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-059</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="150" customHeight="1">
       <c r="A33" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-060</t>
+          <t>MS-CFG-017</t>
         </is>
       </c>
       <c r="B33" s="25" t="inlineStr">
@@ -5995,7 +6156,7 @@
       </c>
       <c r="P33" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-060 홀로그램 스티커 supports size and quantity selection through to cart</t>
+          <t>MS-CFG-017 홀로그램 스티커 supports size and quantity selection through to cart</t>
         </is>
       </c>
       <c r="Q33" s="25" t="inlineStr">
@@ -6020,11 +6181,16 @@
       <c r="V33" s="15" t="n"/>
       <c r="W33" s="15" t="n"/>
       <c r="X33" s="15" t="n"/>
+      <c r="Y33" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-060</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="150" customHeight="1">
       <c r="A34" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-061</t>
+          <t>MS-CFG-018</t>
         </is>
       </c>
       <c r="B34" s="25" t="inlineStr">
@@ -6104,7 +6270,7 @@
       </c>
       <c r="P34" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-061 투명 롤 스티커 supports size and quantity selection through to cart</t>
+          <t>MS-CFG-018 투명 롤 스티커 supports size and quantity selection through to cart</t>
         </is>
       </c>
       <c r="Q34" s="25" t="inlineStr">
@@ -6129,11 +6295,16 @@
       <c r="V34" s="15" t="n"/>
       <c r="W34" s="15" t="n"/>
       <c r="X34" s="15" t="n"/>
+      <c r="Y34" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-061</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="150" customHeight="1">
       <c r="A35" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-062</t>
+          <t>MS-CFG-019</t>
         </is>
       </c>
       <c r="B35" s="25" t="inlineStr">
@@ -6212,7 +6383,7 @@
       </c>
       <c r="P35" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-062 circle sticker: custom individual size recalculates the price</t>
+          <t>MS-CFG-019 circle sticker: custom individual size recalculates the price</t>
         </is>
       </c>
       <c r="Q35" s="25" t="inlineStr">
@@ -6237,11 +6408,16 @@
       <c r="V35" s="15" t="n"/>
       <c r="W35" s="15" t="n"/>
       <c r="X35" s="15" t="n"/>
+      <c r="Y35" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-062</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="150" customHeight="1">
       <c r="A36" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-063</t>
+          <t>MS-CFG-020</t>
         </is>
       </c>
       <c r="B36" s="25" t="inlineStr">
@@ -6320,7 +6496,7 @@
       </c>
       <c r="P36" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-063 circle roll sticker: custom individual size recalculates the price</t>
+          <t>MS-CFG-020 circle roll sticker: custom individual size recalculates the price</t>
         </is>
       </c>
       <c r="Q36" s="25" t="inlineStr">
@@ -6345,11 +6521,16 @@
       <c r="V36" s="15" t="n"/>
       <c r="W36" s="15" t="n"/>
       <c r="X36" s="15" t="n"/>
+      <c r="Y36" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-063</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="150" customHeight="1">
       <c r="A37" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-064</t>
+          <t>MS-CFG-021</t>
         </is>
       </c>
       <c r="B37" s="25" t="inlineStr">
@@ -6428,7 +6609,7 @@
       </c>
       <c r="P37" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-064 circle sticker: bulk quantity tiers surface a discount that smaller tiers do not</t>
+          <t>MS-CFG-021 circle sticker: bulk quantity tiers surface a discount that smaller tiers do not</t>
         </is>
       </c>
       <c r="Q37" s="25" t="inlineStr">
@@ -6453,11 +6634,16 @@
       <c r="V37" s="15" t="n"/>
       <c r="W37" s="15" t="n"/>
       <c r="X37" s="15" t="n"/>
+      <c r="Y37" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-064</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="150" customHeight="1">
       <c r="A38" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-065</t>
+          <t>MS-CFG-022</t>
         </is>
       </c>
       <c r="B38" s="25" t="inlineStr">
@@ -6536,7 +6722,7 @@
       </c>
       <c r="P38" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-065 circle roll sticker: bulk quantity tiers surface a discount that smaller tiers do not</t>
+          <t>MS-CFG-022 circle roll sticker: bulk quantity tiers surface a discount that smaller tiers do not</t>
         </is>
       </c>
       <c r="Q38" s="25" t="inlineStr">
@@ -6561,11 +6747,16 @@
       <c r="V38" s="15" t="n"/>
       <c r="W38" s="15" t="n"/>
       <c r="X38" s="15" t="n"/>
+      <c r="Y38" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-065</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="150" customHeight="1">
       <c r="A39" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-070</t>
+          <t>MS-CFG-023</t>
         </is>
       </c>
       <c r="B39" s="25" t="inlineStr">
@@ -6647,7 +6838,7 @@
       </c>
       <c r="P39" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-070 custom sheet sticker supports material, sheet size, and quantity selection through to cart</t>
+          <t>MS-CFG-023 custom sheet sticker supports material, sheet size, and quantity selection through to cart</t>
         </is>
       </c>
       <c r="Q39" s="25" t="inlineStr">
@@ -6672,11 +6863,16 @@
       <c r="V39" s="15" t="n"/>
       <c r="W39" s="15" t="n"/>
       <c r="X39" s="15" t="n"/>
+      <c r="Y39" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-070</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="150" customHeight="1">
       <c r="A40" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-071</t>
+          <t>MS-CFG-024</t>
         </is>
       </c>
       <c r="B40" s="25" t="inlineStr">
@@ -6757,7 +6953,7 @@
       </c>
       <c r="P40" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-071 lettering sticker supports color, custom text, and quantity selection through to cart</t>
+          <t>MS-CFG-024 lettering sticker supports color, custom text, and quantity selection through to cart</t>
         </is>
       </c>
       <c r="Q40" s="25" t="inlineStr">
@@ -6782,11 +6978,16 @@
       <c r="V40" s="15" t="n"/>
       <c r="W40" s="15" t="n"/>
       <c r="X40" s="15" t="n"/>
+      <c r="Y40" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-071</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="150" customHeight="1">
       <c r="A41" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-072</t>
+          <t>MS-CFG-025</t>
         </is>
       </c>
       <c r="B41" s="25" t="inlineStr">
@@ -6867,7 +7068,7 @@
       </c>
       <c r="P41" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-072 full-color lettering (transfer) sticker supports color, size, and quantity selection through to cart</t>
+          <t>MS-CFG-025 full-color lettering (transfer) sticker supports color, size, and quantity selection through to cart</t>
         </is>
       </c>
       <c r="Q41" s="25" t="inlineStr">
@@ -6892,11 +7093,16 @@
       <c r="V41" s="15" t="n"/>
       <c r="W41" s="15" t="n"/>
       <c r="X41" s="15" t="n"/>
+      <c r="Y41" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-072</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="150" customHeight="1">
       <c r="A42" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-073</t>
+          <t>MS-SHT-001</t>
         </is>
       </c>
       <c r="B42" s="25" t="inlineStr">
@@ -6976,7 +7182,7 @@
       </c>
       <c r="P42" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-073 원형 판스티커 rejects a custom size that fits only one sticker per sheet</t>
+          <t>MS-SHT-001 원형 판스티커 rejects a custom size that fits only one sticker per sheet</t>
         </is>
       </c>
       <c r="Q42" s="25" t="inlineStr">
@@ -7001,11 +7207,16 @@
       <c r="V42" s="15" t="n"/>
       <c r="W42" s="15" t="n"/>
       <c r="X42" s="15" t="n"/>
+      <c r="Y42" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-073</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="150" customHeight="1">
       <c r="A43" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-074</t>
+          <t>MS-SHT-002</t>
         </is>
       </c>
       <c r="B43" s="25" t="inlineStr">
@@ -7084,7 +7295,7 @@
       </c>
       <c r="P43" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-074 circle sheet sticker: the 138x97 gate is exact</t>
+          <t>MS-SHT-002 circle sheet sticker: the 138x97 gate is exact</t>
         </is>
       </c>
       <c r="Q43" s="25" t="inlineStr">
@@ -7109,11 +7320,16 @@
       <c r="V43" s="15" t="n"/>
       <c r="W43" s="15" t="n"/>
       <c r="X43" s="15" t="n"/>
+      <c r="Y43" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-074</t>
+        </is>
+      </c>
     </row>
     <row r="44" ht="150" customHeight="1">
       <c r="A44" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-075</t>
+          <t>MS-SHT-003</t>
         </is>
       </c>
       <c r="B44" s="25" t="inlineStr">
@@ -7192,7 +7408,7 @@
       </c>
       <c r="P44" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-075 원형 판스티커 preset sizes match the shape family table and all fit at least two per sheet</t>
+          <t>MS-SHT-003 원형 판스티커 preset sizes match the shape family table and all fit at least two per sheet</t>
         </is>
       </c>
       <c r="Q44" s="25" t="inlineStr">
@@ -7217,11 +7433,16 @@
       <c r="V44" s="15" t="n"/>
       <c r="W44" s="15" t="n"/>
       <c r="X44" s="15" t="n"/>
+      <c r="Y44" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-075</t>
+        </is>
+      </c>
     </row>
     <row r="45" ht="150" customHeight="1">
       <c r="A45" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-076</t>
+          <t>MS-SHT-004</t>
         </is>
       </c>
       <c r="B45" s="25" t="inlineStr">
@@ -7302,7 +7523,7 @@
       </c>
       <c r="P45" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-076 circle sheet sticker: both cart edit dialogs reject a one-per-sheet custom size</t>
+          <t>MS-SHT-004 circle sheet sticker: both cart edit dialogs reject a one-per-sheet custom size</t>
         </is>
       </c>
       <c r="Q45" s="25" t="inlineStr">
@@ -7327,11 +7548,16 @@
       <c r="V45" s="15" t="n"/>
       <c r="W45" s="15" t="n"/>
       <c r="X45" s="15" t="n"/>
+      <c r="Y45" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-076</t>
+        </is>
+      </c>
     </row>
     <row r="46" ht="150" customHeight="1">
       <c r="A46" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-077</t>
+          <t>MS-SHT-005</t>
         </is>
       </c>
       <c r="B46" s="25" t="inlineStr">
@@ -7410,7 +7636,7 @@
       </c>
       <c r="P46" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-077 circle sheet sticker: the A5 배치 가이드 modal rejects a one-per-sheet custom size</t>
+          <t>MS-SHT-005 circle sheet sticker: the A5 배치 가이드 modal rejects a one-per-sheet custom size</t>
         </is>
       </c>
       <c r="Q46" s="25" t="inlineStr">
@@ -7435,11 +7661,16 @@
       <c r="V46" s="15" t="n"/>
       <c r="W46" s="15" t="n"/>
       <c r="X46" s="15" t="n"/>
+      <c r="Y46" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-077</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="150" customHeight="1">
       <c r="A47" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-078</t>
+          <t>MS-SHT-006</t>
         </is>
       </c>
       <c r="B47" s="25" t="inlineStr">
@@ -7517,7 +7748,7 @@
       </c>
       <c r="P47" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-078 circle sheet sticker: 138x97 packs 2 per sheet and is orderable</t>
+          <t>MS-SHT-006 circle sheet sticker: 138x97 packs 2 per sheet and is orderable</t>
         </is>
       </c>
       <c r="Q47" s="25" t="inlineStr">
@@ -7530,7 +7761,7 @@
       </c>
       <c r="S47" s="25" t="inlineStr">
         <is>
-          <t>The minimum-two-per-sheet error is matched with the regex /한 시트에 최소 2개의 스티커/, the clause shared by both current wordings: the axis-specific line ("...들어가도록 세로 길이를 97mm 이하로 입력해 주세요.", on production since 2026-08-31, shown when only the height is over) and the original generic line ("더 작은 사이즈를 입력해 주세요. 한 시트에 최소 2개의 스티커가 들어가야 합니다.", shown when the width is over). test-case.md still quotes only the old generic literal. The old-literal assertions noted in memory have already been replaced in code by this shared-clause regex. Both gate axes are covered: width (138 vs 139) and height (97 vs 98). test-case.md says rejected sizes fall back to the last valid size (the default 소형); since 2026-08-31 the readout reports the rejected size itself (see MS-V2-073), but this test does not check counts for rejected sizes. test-case.md shows no @production tag for this ID, but the code has it.</t>
+          <t>The minimum-two-per-sheet error is matched with the regex /한 시트에 최소 2개의 스티커/, the clause shared by both current wordings: the axis-specific line ("...들어가도록 세로 길이를 97mm 이하로 입력해 주세요.", on production since 2026-08-31, shown when only the height is over) and the original generic line ("더 작은 사이즈를 입력해 주세요. 한 시트에 최소 2개의 스티커가 들어가야 합니다.", shown when the width is over). test-case.md still quotes only the old generic literal. The old-literal assertions noted in memory have already been replaced in code by this shared-clause regex. Both gate axes are covered: width (138 vs 139) and height (97 vs 98). test-case.md says rejected sizes fall back to the last valid size (the default 소형); since 2026-08-31 the readout reports the rejected size itself (see MS-SHT-001), but this test does not check counts for rejected sizes. test-case.md shows no @production tag for this ID, but the code has it.</t>
         </is>
       </c>
       <c r="T47" s="14" t="inlineStr">
@@ -7542,11 +7773,16 @@
       <c r="V47" s="15" t="n"/>
       <c r="W47" s="15" t="n"/>
       <c r="X47" s="15" t="n"/>
+      <c r="Y47" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-078</t>
+        </is>
+      </c>
     </row>
     <row r="48" ht="150" customHeight="1">
       <c r="A48" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-100</t>
+          <t>MS-CRT-001</t>
         </is>
       </c>
       <c r="B48" s="25" t="inlineStr">
@@ -7627,7 +7863,7 @@
       </c>
       <c r="P48" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-100 removing the only line item leaves an empty cart, not a broken one</t>
+          <t>MS-CRT-001 removing the only line item leaves an empty cart, not a broken one</t>
         </is>
       </c>
       <c r="Q48" s="25" t="inlineStr">
@@ -7652,11 +7888,16 @@
       <c r="V48" s="15" t="n"/>
       <c r="W48" s="15" t="n"/>
       <c r="X48" s="15" t="n"/>
+      <c r="Y48" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-100</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="150" customHeight="1">
       <c r="A49" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-101</t>
+          <t>MS-CRT-002</t>
         </is>
       </c>
       <c r="B49" s="25" t="inlineStr">
@@ -7736,7 +7977,7 @@
       </c>
       <c r="P49" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-101 two distinct products become two lines whose prices sum to the cart total</t>
+          <t>MS-CRT-002 two distinct products become two lines whose prices sum to the cart total</t>
         </is>
       </c>
       <c r="Q49" s="25" t="inlineStr">
@@ -7761,11 +8002,16 @@
       <c r="V49" s="15" t="n"/>
       <c r="W49" s="15" t="n"/>
       <c r="X49" s="15" t="n"/>
+      <c r="Y49" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-101</t>
+        </is>
+      </c>
     </row>
     <row r="50" ht="150" customHeight="1">
       <c r="A50" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-102</t>
+          <t>MS-CRT-003</t>
         </is>
       </c>
       <c r="B50" s="25" t="inlineStr">
@@ -7845,7 +8091,7 @@
       </c>
       <c r="P50" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-102 a guest cart survives a full page reload @smoke</t>
+          <t>MS-CRT-003 a guest cart survives a full page reload @smoke</t>
         </is>
       </c>
       <c r="Q50" s="25" t="inlineStr">
@@ -7870,11 +8116,16 @@
       <c r="V50" s="15" t="n"/>
       <c r="W50" s="15" t="n"/>
       <c r="X50" s="15" t="n"/>
+      <c r="Y50" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-102</t>
+        </is>
+      </c>
     </row>
     <row r="51" ht="150" customHeight="1">
       <c r="A51" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-103</t>
+          <t>MS-CRT-004</t>
         </is>
       </c>
       <c r="B51" s="25" t="inlineStr">
@@ -7954,7 +8205,7 @@
       </c>
       <c r="P51" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-103 the cart page confirms a removal before acting on it</t>
+          <t>MS-CRT-004 the cart page confirms a removal before acting on it</t>
         </is>
       </c>
       <c r="Q51" s="25" t="inlineStr">
@@ -7979,11 +8230,16 @@
       <c r="V51" s="15" t="n"/>
       <c r="W51" s="15" t="n"/>
       <c r="X51" s="15" t="n"/>
+      <c r="Y51" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-103</t>
+        </is>
+      </c>
     </row>
     <row r="52" ht="150" customHeight="1">
       <c r="A52" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-104</t>
+          <t>MS-CRT-005</t>
         </is>
       </c>
       <c r="B52" s="25" t="inlineStr">
@@ -8063,7 +8319,7 @@
       </c>
       <c r="P52" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-104 a guest cart is merged into the member cart on login</t>
+          <t>MS-CRT-005 a guest cart is merged into the member cart on login</t>
         </is>
       </c>
       <c r="Q52" s="25" t="inlineStr">
@@ -8088,11 +8344,16 @@
       <c r="V52" s="15" t="n"/>
       <c r="W52" s="15" t="n"/>
       <c r="X52" s="15" t="n"/>
+      <c r="Y52" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-104</t>
+        </is>
+      </c>
     </row>
     <row r="53" ht="150" customHeight="1">
       <c r="A53" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-105</t>
+          <t>MS-CRT-006</t>
         </is>
       </c>
       <c r="B53" s="25" t="inlineStr">
@@ -8170,7 +8431,7 @@
       </c>
       <c r="P53" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-105 an empty cart page offers a way back into the catalog</t>
+          <t>MS-CRT-006 an empty cart page offers a way back into the catalog</t>
         </is>
       </c>
       <c r="Q53" s="25" t="inlineStr">
@@ -8195,11 +8456,16 @@
       <c r="V53" s="15" t="n"/>
       <c r="W53" s="15" t="n"/>
       <c r="X53" s="15" t="n"/>
+      <c r="Y53" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-105</t>
+        </is>
+      </c>
     </row>
     <row r="54" ht="150" customHeight="1">
       <c r="A54" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-025</t>
+          <t>MS-CHK-001</t>
         </is>
       </c>
       <c r="B54" s="25" t="inlineStr">
@@ -8282,7 +8548,7 @@
       </c>
       <c r="P54" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-025 guest checkout completes via the KakaoPay sandbox and sends an order-confirmation email</t>
+          <t>MS-CHK-001 guest checkout completes via the KakaoPay sandbox and sends an order-confirmation email</t>
         </is>
       </c>
       <c r="Q54" s="25" t="inlineStr">
@@ -8307,11 +8573,16 @@
       <c r="V54" s="15" t="n"/>
       <c r="W54" s="15" t="n"/>
       <c r="X54" s="15" t="n"/>
+      <c r="Y54" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-025</t>
+        </is>
+      </c>
     </row>
     <row r="55" ht="150" customHeight="1">
       <c r="A55" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-041</t>
+          <t>MS-CHK-002</t>
         </is>
       </c>
       <c r="B55" s="25" t="inlineStr">
@@ -8389,7 +8660,7 @@
       </c>
       <c r="P55" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-041 checkout page renders shipping, payment, and order summary without submitting</t>
+          <t>MS-CHK-002 checkout page renders shipping, payment, and order summary without submitting</t>
         </is>
       </c>
       <c r="Q55" s="25" t="inlineStr">
@@ -8414,11 +8685,16 @@
       <c r="V55" s="15" t="n"/>
       <c r="W55" s="15" t="n"/>
       <c r="X55" s="15" t="n"/>
+      <c r="Y55" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-041</t>
+        </is>
+      </c>
     </row>
     <row r="56" ht="150" customHeight="1">
       <c r="A56" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-042</t>
+          <t>MS-CHK-003</t>
         </is>
       </c>
       <c r="B56" s="25" t="inlineStr">
@@ -8496,7 +8772,7 @@
       </c>
       <c r="P56" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-042 checkout blocks payment submission when required fields are blank</t>
+          <t>MS-CHK-003 checkout blocks payment submission when required fields are blank</t>
         </is>
       </c>
       <c r="Q56" s="25" t="inlineStr">
@@ -8521,11 +8797,16 @@
       <c r="V56" s="15" t="n"/>
       <c r="W56" s="15" t="n"/>
       <c r="X56" s="15" t="n"/>
+      <c r="Y56" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-042</t>
+        </is>
+      </c>
     </row>
     <row r="57" ht="150" customHeight="1">
       <c r="A57" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-097</t>
+          <t>MS-CHK-004</t>
         </is>
       </c>
       <c r="B57" s="25" t="inlineStr">
@@ -8605,7 +8886,7 @@
       </c>
       <c r="P57" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-097 the quoted price survives product page, cart, and checkout unchanged</t>
+          <t>MS-CHK-004 the quoted price survives product page, cart, and checkout unchanged</t>
         </is>
       </c>
       <c r="Q57" s="25" t="inlineStr">
@@ -8630,11 +8911,16 @@
       <c r="V57" s="15" t="n"/>
       <c r="W57" s="15" t="n"/>
       <c r="X57" s="15" t="n"/>
+      <c r="Y57" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-097</t>
+        </is>
+      </c>
     </row>
     <row r="58" ht="150" customHeight="1">
       <c r="A58" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-098</t>
+          <t>MS-CHK-005</t>
         </is>
       </c>
       <c r="B58" s="25" t="inlineStr">
@@ -8713,7 +8999,7 @@
       </c>
       <c r="P58" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-098 an order below the free-shipping threshold is charged shipping</t>
+          <t>MS-CHK-005 an order below the free-shipping threshold is charged shipping</t>
         </is>
       </c>
       <c r="Q58" s="25" t="inlineStr">
@@ -8738,11 +9024,16 @@
       <c r="V58" s="15" t="n"/>
       <c r="W58" s="15" t="n"/>
       <c r="X58" s="15" t="n"/>
+      <c r="Y58" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-098</t>
+        </is>
+      </c>
     </row>
     <row r="59" ht="150" customHeight="1">
       <c r="A59" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-099</t>
+          <t>MS-CHK-006</t>
         </is>
       </c>
       <c r="B59" s="25" t="inlineStr">
@@ -8821,7 +9112,7 @@
       </c>
       <c r="P59" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-099 an order at or above the free-shipping threshold ships free</t>
+          <t>MS-CHK-006 an order at or above the free-shipping threshold ships free</t>
         </is>
       </c>
       <c r="Q59" s="25" t="inlineStr">
@@ -8846,6 +9137,11 @@
       <c r="V59" s="15" t="n"/>
       <c r="W59" s="15" t="n"/>
       <c r="X59" s="15" t="n"/>
+      <c r="Y59" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-099</t>
+        </is>
+      </c>
     </row>
     <row r="60" ht="150" customHeight="1">
       <c r="A60" s="12" t="inlineStr">
@@ -11910,7 +12206,7 @@
     <row r="88" ht="150" customHeight="1">
       <c r="A88" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-026</t>
+          <t>MS-AUTH-001</t>
         </is>
       </c>
       <c r="B88" s="25" t="inlineStr">
@@ -11988,7 +12284,7 @@
       </c>
       <c r="P88" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-026 account navigation opens login</t>
+          <t>MS-AUTH-001 account navigation opens login</t>
         </is>
       </c>
       <c r="Q88" s="25" t="inlineStr">
@@ -12013,11 +12309,16 @@
       <c r="V88" s="15" t="n"/>
       <c r="W88" s="15" t="n"/>
       <c r="X88" s="15" t="n"/>
+      <c r="Y88" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-026</t>
+        </is>
+      </c>
     </row>
     <row r="89" ht="150" customHeight="1">
       <c r="A89" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-027</t>
+          <t>MS-AUTH-002</t>
         </is>
       </c>
       <c r="B89" s="25" t="inlineStr">
@@ -12094,7 +12395,7 @@
       </c>
       <c r="P89" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-027 member login form exposes expected controls</t>
+          <t>MS-AUTH-002 member login form exposes expected controls</t>
         </is>
       </c>
       <c r="Q89" s="25" t="inlineStr">
@@ -12119,11 +12420,16 @@
       <c r="V89" s="15" t="n"/>
       <c r="W89" s="15" t="n"/>
       <c r="X89" s="15" t="n"/>
+      <c r="Y89" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-027</t>
+        </is>
+      </c>
     </row>
     <row r="90" ht="150" customHeight="1">
       <c r="A90" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-028</t>
+          <t>MS-AUTH-003</t>
         </is>
       </c>
       <c r="B90" s="25" t="inlineStr">
@@ -12200,7 +12506,7 @@
       </c>
       <c r="P90" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-028 blank login is blocked before the auth endpoint is called @validation</t>
+          <t>MS-AUTH-003 blank login is blocked before the auth endpoint is called @validation</t>
         </is>
       </c>
       <c r="Q90" s="25" t="inlineStr">
@@ -12225,11 +12531,16 @@
       <c r="V90" s="15" t="n"/>
       <c r="W90" s="15" t="n"/>
       <c r="X90" s="15" t="n"/>
+      <c r="Y90" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-028</t>
+        </is>
+      </c>
     </row>
     <row r="91" ht="150" customHeight="1">
       <c r="A91" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-029</t>
+          <t>MS-AUTH-004</t>
         </is>
       </c>
       <c r="B91" s="25" t="inlineStr">
@@ -12306,7 +12617,7 @@
       </c>
       <c r="P91" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-029 malformed email is rejected without starting an auth session @validation</t>
+          <t>MS-AUTH-004 malformed email is rejected without starting an auth session @validation</t>
         </is>
       </c>
       <c r="Q91" s="25" t="inlineStr">
@@ -12327,11 +12638,16 @@
       <c r="V91" s="15" t="n"/>
       <c r="W91" s="15" t="n"/>
       <c r="X91" s="15" t="n"/>
+      <c r="Y91" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-029</t>
+        </is>
+      </c>
     </row>
     <row r="92" ht="150" customHeight="1">
       <c r="A92" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-030</t>
+          <t>MS-AUTH-005</t>
         </is>
       </c>
       <c r="B92" s="25" t="inlineStr">
@@ -12410,7 +12726,7 @@
       </c>
       <c r="P92" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-030 invalid credentials fail safely and keep the user anonymous @validation</t>
+          <t>MS-AUTH-005 invalid credentials fail safely and keep the user anonymous @validation</t>
         </is>
       </c>
       <c r="Q92" s="25" t="inlineStr">
@@ -12435,11 +12751,16 @@
       <c r="V92" s="15" t="n"/>
       <c r="W92" s="15" t="n"/>
       <c r="X92" s="15" t="n"/>
+      <c r="Y92" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-030</t>
+        </is>
+      </c>
     </row>
     <row r="93" ht="150" customHeight="1">
       <c r="A93" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-031</t>
+          <t>MS-AUTH-006</t>
         </is>
       </c>
       <c r="B93" s="25" t="inlineStr">
@@ -12519,7 +12840,7 @@
       </c>
       <c r="P93" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-031 password visibility toggle masks and unmasks password</t>
+          <t>MS-AUTH-006 password visibility toggle masks and unmasks password</t>
         </is>
       </c>
       <c r="Q93" s="25" t="inlineStr">
@@ -12532,7 +12853,7 @@
       </c>
       <c r="S93" s="25" t="inlineStr">
         <is>
-          <t>Also covers MS-V2-044 (re-verification against production on 2026-08-11), which has no separate test; the 2026-08-10 toggle bug in test-case.md is no longer reproducible and the test is no longer fixme'd. Page load already round-trips the toggle once to detect hydration. test-case.md lists @regression; the spec does not carry it.</t>
+          <t>Also covers MS-AUTH-011 (re-verification against production on 2026-08-11), which has no separate test; the 2026-08-10 toggle bug in test-case.md is no longer reproducible and the test is no longer fixme'd. Page load already round-trips the toggle once to detect hydration. test-case.md lists @regression; the spec does not carry it.</t>
         </is>
       </c>
       <c r="T93" s="14" t="inlineStr">
@@ -12544,11 +12865,16 @@
       <c r="V93" s="15" t="n"/>
       <c r="W93" s="15" t="n"/>
       <c r="X93" s="15" t="n"/>
+      <c r="Y93" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-031</t>
+        </is>
+      </c>
     </row>
     <row r="94" ht="150" customHeight="1">
       <c r="A94" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-032</t>
+          <t>MS-AUTH-007</t>
         </is>
       </c>
       <c r="B94" s="25" t="inlineStr">
@@ -12627,7 +12953,7 @@
       </c>
       <c r="P94" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-032 forgot-password recovery opens and validates its email input @validation</t>
+          <t>MS-AUTH-007 forgot-password recovery opens and validates its email input @validation</t>
         </is>
       </c>
       <c r="Q94" s="25" t="inlineStr">
@@ -12640,7 +12966,7 @@
       </c>
       <c r="S94" s="25" t="inlineStr">
         <is>
-          <t>Unlike MS-V2-028/029, the code does not watch the network, so the claim that no recovery request is sent is not actually verified. Never submit a real address in production.</t>
+          <t>Unlike MS-AUTH-003/MS-AUTH-004, the code does not watch the network, so the claim that no recovery request is sent is not actually verified. Never submit a real address in production.</t>
         </is>
       </c>
       <c r="T94" s="14" t="inlineStr">
@@ -12652,11 +12978,16 @@
       <c r="V94" s="15" t="n"/>
       <c r="W94" s="15" t="n"/>
       <c r="X94" s="15" t="n"/>
+      <c r="Y94" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-032</t>
+        </is>
+      </c>
     </row>
     <row r="95" ht="150" customHeight="1">
       <c r="A95" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-033</t>
+          <t>MS-AUTH-008</t>
         </is>
       </c>
       <c r="B95" s="25" t="inlineStr">
@@ -12733,7 +13064,7 @@
       </c>
       <c r="P95" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-033 register entry is reachable from login</t>
+          <t>MS-AUTH-008 register entry is reachable from login</t>
         </is>
       </c>
       <c r="Q95" s="25" t="inlineStr">
@@ -12746,7 +13077,7 @@
       </c>
       <c r="S95" s="25" t="inlineStr">
         <is>
-          <t>test-case.md steps 4-6 (check registration fields, go back, login form restored) are not in this test; register controls are MS-V2-079 and the return trip is MS-V2-085. Nothing is submitted.</t>
+          <t>test-case.md steps 4-6 (check registration fields, go back, login form restored) are not in this test; register controls are MS-AUTH-012 and the return trip is MS-AUTH-018. Nothing is submitted.</t>
         </is>
       </c>
       <c r="T95" s="14" t="inlineStr">
@@ -12758,11 +13089,16 @@
       <c r="V95" s="15" t="n"/>
       <c r="W95" s="15" t="n"/>
       <c r="X95" s="15" t="n"/>
+      <c r="Y95" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-033</t>
+        </is>
+      </c>
     </row>
     <row r="96" ht="150" customHeight="1">
       <c r="A96" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-034</t>
+          <t>MS-AUTH-009</t>
         </is>
       </c>
       <c r="B96" s="25" t="inlineStr">
@@ -12840,7 +13176,7 @@
       </c>
       <c r="P96" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-034 seeded member can log in @credentialed</t>
+          <t>MS-AUTH-009 seeded member can log in @credentialed</t>
         </is>
       </c>
       <c r="Q96" s="25" t="inlineStr">
@@ -12865,11 +13201,16 @@
       <c r="V96" s="15" t="n"/>
       <c r="W96" s="15" t="n"/>
       <c r="X96" s="15" t="n"/>
+      <c r="Y96" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-034</t>
+        </is>
+      </c>
     </row>
     <row r="97" ht="150" customHeight="1">
       <c r="A97" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-035</t>
+          <t>MS-AUTH-010</t>
         </is>
       </c>
       <c r="B97" s="25" t="inlineStr">
@@ -12949,7 +13290,7 @@
       </c>
       <c r="P97" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-035 session persists across reload and navigation, and logout clears it @credentialed</t>
+          <t>MS-AUTH-010 session persists across reload and navigation, and logout clears it @credentialed</t>
         </is>
       </c>
       <c r="Q97" s="25" t="inlineStr">
@@ -12974,11 +13315,16 @@
       <c r="V97" s="15" t="n"/>
       <c r="W97" s="15" t="n"/>
       <c r="X97" s="15" t="n"/>
+      <c r="Y97" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-035</t>
+        </is>
+      </c>
     </row>
     <row r="98" ht="150" customHeight="1">
       <c r="A98" s="16" t="inlineStr">
         <is>
-          <t>MS-V2-044</t>
+          <t>MS-AUTH-011</t>
         </is>
       </c>
       <c r="B98" s="25" t="inlineStr">
@@ -12998,7 +13344,7 @@
       </c>
       <c r="E98" s="17" t="inlineStr">
         <is>
-          <t>Withdrawn: re-verification of the MS-V2-031 password visibility toggle. Merged into MS-V2-031.</t>
+          <t>Withdrawn: re-verification of the MS-AUTH-006 password visibility toggle. Merged into MS-AUTH-006.</t>
         </is>
       </c>
       <c r="F98" s="13" t="inlineStr">
@@ -13066,7 +13412,7 @@
       </c>
       <c r="S98" s="25" t="inlineStr">
         <is>
-          <t>withdrawn 2026-08-11: the production toggle bug (rendered but did not unmask) no longer reproduced, so the re-verification was folded into MS-V2-031 (see the comment in tests/e2e/storefront/auth/login.spec.ts). Keep the ID; do not reuse it.</t>
+          <t>withdrawn 2026-08-11: the production toggle bug (rendered but did not unmask) no longer reproduced, so the re-verification was folded into MS-AUTH-006 (see the comment in tests/e2e/storefront/auth/login.spec.ts). Keep the ID; do not reuse it.</t>
         </is>
       </c>
       <c r="T98" s="14" t="inlineStr">
@@ -13078,11 +13424,16 @@
       <c r="V98" s="15" t="n"/>
       <c r="W98" s="15" t="n"/>
       <c r="X98" s="15" t="n"/>
+      <c r="Y98" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-044</t>
+        </is>
+      </c>
     </row>
     <row r="99" ht="150" customHeight="1">
       <c r="A99" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-079</t>
+          <t>MS-AUTH-012</t>
         </is>
       </c>
       <c r="B99" s="25" t="inlineStr">
@@ -13160,7 +13511,7 @@
       </c>
       <c r="P99" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-079 register form exposes expected controls @smoke</t>
+          <t>MS-AUTH-012 register form exposes expected controls @smoke</t>
         </is>
       </c>
       <c r="Q99" s="25" t="inlineStr">
@@ -13185,11 +13536,16 @@
       <c r="V99" s="15" t="n"/>
       <c r="W99" s="15" t="n"/>
       <c r="X99" s="15" t="n"/>
+      <c r="Y99" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-079</t>
+        </is>
+      </c>
     </row>
     <row r="100" ht="150" customHeight="1">
       <c r="A100" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-080</t>
+          <t>MS-AUTH-013</t>
         </is>
       </c>
       <c r="B100" s="25" t="inlineStr">
@@ -13266,7 +13622,7 @@
       </c>
       <c r="P100" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-080 blank register submit is blocked with required-field validation @validation</t>
+          <t>MS-AUTH-013 blank register submit is blocked with required-field validation @validation</t>
         </is>
       </c>
       <c r="Q100" s="25" t="inlineStr">
@@ -13291,11 +13647,16 @@
       <c r="V100" s="15" t="n"/>
       <c r="W100" s="15" t="n"/>
       <c r="X100" s="15" t="n"/>
+      <c r="Y100" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-080</t>
+        </is>
+      </c>
     </row>
     <row r="101" ht="150" customHeight="1">
       <c r="A101" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-081</t>
+          <t>MS-AUTH-014</t>
         </is>
       </c>
       <c r="B101" s="25" t="inlineStr">
@@ -13372,7 +13733,7 @@
       </c>
       <c r="P101" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-081 malformed email is rejected before any account is requested @validation</t>
+          <t>MS-AUTH-014 malformed email is rejected before any account is requested @validation</t>
         </is>
       </c>
       <c r="Q101" s="25" t="inlineStr">
@@ -13385,7 +13746,7 @@
       </c>
       <c r="S101" s="25" t="inlineStr">
         <is>
-          <t>URL is not asserted here (unlike MS-V2-080).</t>
+          <t>URL is not asserted here (unlike MS-AUTH-013).</t>
         </is>
       </c>
       <c r="T101" s="14" t="inlineStr">
@@ -13397,11 +13758,16 @@
       <c r="V101" s="15" t="n"/>
       <c r="W101" s="15" t="n"/>
       <c r="X101" s="15" t="n"/>
+      <c r="Y101" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-081</t>
+        </is>
+      </c>
     </row>
     <row r="102" ht="150" customHeight="1">
       <c r="A102" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-082</t>
+          <t>MS-AUTH-015</t>
         </is>
       </c>
       <c r="B102" s="25" t="inlineStr">
@@ -13478,7 +13844,7 @@
       </c>
       <c r="P102" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-082 password below the stated policy is rejected @validation</t>
+          <t>MS-AUTH-015 password below the stated policy is rejected @validation</t>
         </is>
       </c>
       <c r="Q102" s="25" t="inlineStr">
@@ -13503,11 +13869,16 @@
       <c r="V102" s="15" t="n"/>
       <c r="W102" s="15" t="n"/>
       <c r="X102" s="15" t="n"/>
+      <c r="Y102" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-082</t>
+        </is>
+      </c>
     </row>
     <row r="103" ht="150" customHeight="1">
       <c r="A103" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-083</t>
+          <t>MS-AUTH-016</t>
         </is>
       </c>
       <c r="B103" s="25" t="inlineStr">
@@ -13585,7 +13956,7 @@
       </c>
       <c r="P103" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-083 registration is blocked until the terms checkbox is agreed @validation</t>
+          <t>MS-AUTH-016 registration is blocked until the terms checkbox is agreed @validation</t>
         </is>
       </c>
       <c r="Q103" s="25" t="inlineStr">
@@ -13610,11 +13981,16 @@
       <c r="V103" s="15" t="n"/>
       <c r="W103" s="15" t="n"/>
       <c r="X103" s="15" t="n"/>
+      <c r="Y103" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-083</t>
+        </is>
+      </c>
     </row>
     <row r="104" ht="150" customHeight="1">
       <c r="A104" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-084</t>
+          <t>MS-AUTH-017</t>
         </is>
       </c>
       <c r="B104" s="25" t="inlineStr">
@@ -13692,7 +14068,7 @@
       </c>
       <c r="P104" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-084 register password visibility toggle masks and unmasks</t>
+          <t>MS-AUTH-017 register password visibility toggle masks and unmasks</t>
         </is>
       </c>
       <c r="Q104" s="25" t="inlineStr">
@@ -13717,11 +14093,16 @@
       <c r="V104" s="15" t="n"/>
       <c r="W104" s="15" t="n"/>
       <c r="X104" s="15" t="n"/>
+      <c r="Y104" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-084</t>
+        </is>
+      </c>
     </row>
     <row r="105" ht="150" customHeight="1">
       <c r="A105" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-085</t>
+          <t>MS-AUTH-018</t>
         </is>
       </c>
       <c r="B105" s="25" t="inlineStr">
@@ -13798,7 +14179,7 @@
       </c>
       <c r="P105" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-085 login entry is reachable from register</t>
+          <t>MS-AUTH-018 login entry is reachable from register</t>
         </is>
       </c>
       <c r="Q105" s="25" t="inlineStr">
@@ -13823,11 +14204,16 @@
       <c r="V105" s="15" t="n"/>
       <c r="W105" s="15" t="n"/>
       <c r="X105" s="15" t="n"/>
+      <c r="Y105" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-085</t>
+        </is>
+      </c>
     </row>
     <row r="106" ht="150" customHeight="1">
       <c r="A106" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-086</t>
+          <t>MS-AUTH-019</t>
         </is>
       </c>
       <c r="B106" s="25" t="inlineStr">
@@ -13905,7 +14291,7 @@
       </c>
       <c r="P106" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-086 registering an existing email offers sign-in instead of a duplicate account @credentialed</t>
+          <t>MS-AUTH-019 registering an existing email offers sign-in instead of a duplicate account @credentialed</t>
         </is>
       </c>
       <c r="Q106" s="25" t="inlineStr">
@@ -13930,11 +14316,16 @@
       <c r="V106" s="15" t="n"/>
       <c r="W106" s="15" t="n"/>
       <c r="X106" s="15" t="n"/>
+      <c r="Y106" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-086</t>
+        </is>
+      </c>
     </row>
     <row r="107" ht="150" customHeight="1">
       <c r="A107" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-087</t>
+          <t>MS-AUTH-020</t>
         </is>
       </c>
       <c r="B107" s="25" t="inlineStr">
@@ -14013,7 +14404,7 @@
       </c>
       <c r="P107" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-087 a wrong verification code is rejected and creates no account</t>
+          <t>MS-AUTH-020 a wrong verification code is rejected and creates no account</t>
         </is>
       </c>
       <c r="Q107" s="25" t="inlineStr">
@@ -14038,11 +14429,16 @@
       <c r="V107" s="15" t="n"/>
       <c r="W107" s="15" t="n"/>
       <c r="X107" s="15" t="n"/>
+      <c r="Y107" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-087</t>
+        </is>
+      </c>
     </row>
     <row r="108" ht="150" customHeight="1">
       <c r="A108" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-088</t>
+          <t>MS-AUTH-021</t>
         </is>
       </c>
       <c r="B108" s="25" t="inlineStr">
@@ -14122,7 +14518,7 @@
       </c>
       <c r="P108" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-088 a correct verification code creates the account and signs the new member in</t>
+          <t>MS-AUTH-021 a correct verification code creates the account and signs the new member in</t>
         </is>
       </c>
       <c r="Q108" s="25" t="inlineStr">
@@ -14135,7 +14531,7 @@
       </c>
       <c r="S108" s="25" t="inlineStr">
         <is>
-          <t>Discrepancy: test-case.md says the account needs no cleanup; the code records it (createdBy MS-V2-088) in .auth/created-accounts.jsonl, and global teardown deletes it only when TEST_DATA_USER_DELETE_ENDPOINT is set. Otherwise teardown warns and the real account stays on the dev server. Carries @production from its describe block but is gated and excluded from prod scripts by @destructive; do not run on production.</t>
+          <t>Discrepancy: test-case.md says the account needs no cleanup; the code records it (createdBy MS-AUTH-021) in .auth/created-accounts.jsonl, and global teardown deletes it only when TEST_DATA_USER_DELETE_ENDPOINT is set. Otherwise teardown warns and the real account stays on the dev server. Carries @production from its describe block but is gated and excluded from prod scripts by @destructive; do not run on production.</t>
         </is>
       </c>
       <c r="T108" s="14" t="inlineStr">
@@ -14147,11 +14543,16 @@
       <c r="V108" s="15" t="n"/>
       <c r="W108" s="15" t="n"/>
       <c r="X108" s="15" t="n"/>
+      <c r="Y108" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-088</t>
+        </is>
+      </c>
     </row>
     <row r="109" ht="150" customHeight="1">
       <c r="A109" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-089</t>
+          <t>MS-AUTH-022</t>
         </is>
       </c>
       <c r="B109" s="25" t="inlineStr">
@@ -14229,7 +14630,7 @@
       </c>
       <c r="P109" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-089 account profile exposes the password change controls @smoke</t>
+          <t>MS-AUTH-022 account profile exposes the password change controls @smoke</t>
         </is>
       </c>
       <c r="Q109" s="25" t="inlineStr">
@@ -14254,11 +14655,16 @@
       <c r="V109" s="15" t="n"/>
       <c r="W109" s="15" t="n"/>
       <c r="X109" s="15" t="n"/>
+      <c r="Y109" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-089</t>
+        </is>
+      </c>
     </row>
     <row r="110" ht="150" customHeight="1">
       <c r="A110" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-090</t>
+          <t>MS-AUTH-023</t>
         </is>
       </c>
       <c r="B110" s="25" t="inlineStr">
@@ -14337,7 +14743,7 @@
       </c>
       <c r="P110" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-090 change password stays disabled until every field is filled @validation</t>
+          <t>MS-AUTH-023 change password stays disabled until every field is filled @validation</t>
         </is>
       </c>
       <c r="Q110" s="25" t="inlineStr">
@@ -14362,11 +14768,16 @@
       <c r="V110" s="15" t="n"/>
       <c r="W110" s="15" t="n"/>
       <c r="X110" s="15" t="n"/>
+      <c r="Y110" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-090</t>
+        </is>
+      </c>
     </row>
     <row r="111" ht="150" customHeight="1">
       <c r="A111" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-091</t>
+          <t>MS-AUTH-024</t>
         </is>
       </c>
       <c r="B111" s="25" t="inlineStr">
@@ -14444,7 +14855,7 @@
       </c>
       <c r="P111" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-091 a mismatched confirmation is rejected @validation</t>
+          <t>MS-AUTH-024 a mismatched confirmation is rejected @validation</t>
         </is>
       </c>
       <c r="Q111" s="25" t="inlineStr">
@@ -14469,11 +14880,16 @@
       <c r="V111" s="15" t="n"/>
       <c r="W111" s="15" t="n"/>
       <c r="X111" s="15" t="n"/>
+      <c r="Y111" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-091</t>
+        </is>
+      </c>
     </row>
     <row r="112" ht="150" customHeight="1">
       <c r="A112" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-092</t>
+          <t>MS-AUTH-025</t>
         </is>
       </c>
       <c r="B112" s="25" t="inlineStr">
@@ -14551,7 +14967,7 @@
       </c>
       <c r="P112" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-092 a new password below the policy is rejected @validation</t>
+          <t>MS-AUTH-025 a new password below the policy is rejected @validation</t>
         </is>
       </c>
       <c r="Q112" s="25" t="inlineStr">
@@ -14576,11 +14992,16 @@
       <c r="V112" s="15" t="n"/>
       <c r="W112" s="15" t="n"/>
       <c r="X112" s="15" t="n"/>
+      <c r="Y112" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-092</t>
+        </is>
+      </c>
     </row>
     <row r="113" ht="150" customHeight="1">
       <c r="A113" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-093</t>
+          <t>MS-AUTH-026</t>
         </is>
       </c>
       <c r="B113" s="25" t="inlineStr">
@@ -14658,7 +15079,7 @@
       </c>
       <c r="P113" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-093 a wrong current password is rejected @validation</t>
+          <t>MS-AUTH-026 a wrong current password is rejected @validation</t>
         </is>
       </c>
       <c r="Q113" s="25" t="inlineStr">
@@ -14683,11 +15104,16 @@
       <c r="V113" s="15" t="n"/>
       <c r="W113" s="15" t="n"/>
       <c r="X113" s="15" t="n"/>
+      <c r="Y113" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-093</t>
+        </is>
+      </c>
     </row>
     <row r="114" ht="150" customHeight="1">
       <c r="A114" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-094</t>
+          <t>MS-AUTH-027</t>
         </is>
       </c>
       <c r="B114" s="25" t="inlineStr">
@@ -14767,7 +15193,7 @@
       </c>
       <c r="P114" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-094 changing a password rotates the credential end to end</t>
+          <t>MS-AUTH-027 changing a password rotates the credential end to end</t>
         </is>
       </c>
       <c r="Q114" s="25" t="inlineStr">
@@ -14780,7 +15206,7 @@
       </c>
       <c r="S114" s="25" t="inlineStr">
         <is>
-          <t>Creates a real member account. It is recorded (createdBy MS-V2-094) in .auth/created-accounts.jsonl; global teardown deletes it only when TEST_DATA_USER_DELETE_ENDPOINT is set, otherwise it just warns and the account stays on the server. Carries @production through its describe block but is skipped unless RUN_AUTH_DESTRUCTIVE_E2E=true and excluded from the prod scripts by @destructive; never run on production. Uses its own account so the seeded member's password is never touched.</t>
+          <t>Creates a real member account. It is recorded (createdBy MS-AUTH-027) in .auth/created-accounts.jsonl; global teardown deletes it only when TEST_DATA_USER_DELETE_ENDPOINT is set, otherwise it just warns and the account stays on the server. Carries @production through its describe block but is skipped unless RUN_AUTH_DESTRUCTIVE_E2E=true and excluded from the prod scripts by @destructive; never run on production. Uses its own account so the seeded member's password is never touched.</t>
         </is>
       </c>
       <c r="T114" s="14" t="inlineStr">
@@ -14792,11 +15218,16 @@
       <c r="V114" s="15" t="n"/>
       <c r="W114" s="15" t="n"/>
       <c r="X114" s="15" t="n"/>
+      <c r="Y114" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-094</t>
+        </is>
+      </c>
     </row>
     <row r="115" ht="150" customHeight="1">
       <c r="A115" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-095</t>
+          <t>MS-AUTH-028</t>
         </is>
       </c>
       <c r="B115" s="25" t="inlineStr">
@@ -14873,7 +15304,7 @@
       </c>
       <c r="P115" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-095 a member-only route is not reachable anonymously</t>
+          <t>MS-AUTH-028 a member-only route is not reachable anonymously</t>
         </is>
       </c>
       <c r="Q115" s="25" t="inlineStr">
@@ -14898,11 +15329,16 @@
       <c r="V115" s="15" t="n"/>
       <c r="W115" s="15" t="n"/>
       <c r="X115" s="15" t="n"/>
+      <c r="Y115" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-095</t>
+        </is>
+      </c>
     </row>
     <row r="116" ht="150" customHeight="1">
       <c r="A116" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-096</t>
+          <t>MS-AUTH-029</t>
         </is>
       </c>
       <c r="B116" s="25" t="inlineStr">
@@ -14979,7 +15415,7 @@
       </c>
       <c r="P116" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-096 non-member mode swaps in the guest order-lookup form</t>
+          <t>MS-AUTH-029 non-member mode swaps in the guest order-lookup form</t>
         </is>
       </c>
       <c r="Q116" s="25" t="inlineStr">
@@ -14992,7 +15428,7 @@
       </c>
       <c r="S116" s="25" t="inlineStr">
         <is>
-          <t>Nothing is submitted; actual lookups are MS-V2-112 to MS-V2-114.</t>
+          <t>Nothing is submitted; actual lookups are MS-AUTH-030 to MS-AUTH-032.</t>
         </is>
       </c>
       <c r="T116" s="14" t="inlineStr">
@@ -15004,11 +15440,16 @@
       <c r="V116" s="15" t="n"/>
       <c r="W116" s="15" t="n"/>
       <c r="X116" s="15" t="n"/>
+      <c r="Y116" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-096</t>
+        </is>
+      </c>
     </row>
     <row r="117" ht="150" customHeight="1">
       <c r="A117" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-112</t>
+          <t>MS-AUTH-030</t>
         </is>
       </c>
       <c r="B117" s="25" t="inlineStr">
@@ -15086,7 +15527,7 @@
       </c>
       <c r="P117" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-112 an unknown order number is refused without signing anyone in</t>
+          <t>MS-AUTH-030 an unknown order number is refused without signing anyone in</t>
         </is>
       </c>
       <c r="Q117" s="25" t="inlineStr">
@@ -15111,11 +15552,16 @@
       <c r="V117" s="15" t="n"/>
       <c r="W117" s="15" t="n"/>
       <c r="X117" s="15" t="n"/>
+      <c r="Y117" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-112</t>
+        </is>
+      </c>
     </row>
     <row r="118" ht="150" customHeight="1">
       <c r="A118" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-113</t>
+          <t>MS-AUTH-031</t>
         </is>
       </c>
       <c r="B118" s="25" t="inlineStr">
@@ -15192,7 +15638,7 @@
       </c>
       <c r="P118" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-113 blank guest lookup is blocked before the endpoint is called @validation</t>
+          <t>MS-AUTH-031 blank guest lookup is blocked before the endpoint is called @validation</t>
         </is>
       </c>
       <c r="Q118" s="25" t="inlineStr">
@@ -15217,11 +15663,16 @@
       <c r="V118" s="15" t="n"/>
       <c r="W118" s="15" t="n"/>
       <c r="X118" s="15" t="n"/>
+      <c r="Y118" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-113</t>
+        </is>
+      </c>
     </row>
     <row r="119" ht="150" customHeight="1">
       <c r="A119" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-114</t>
+          <t>MS-AUTH-032</t>
         </is>
       </c>
       <c r="B119" s="25" t="inlineStr">
@@ -15299,7 +15750,7 @@
       </c>
       <c r="P119" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-114 the refusal does not reveal whether the email belongs to an account @credentialed</t>
+          <t>MS-AUTH-032 the refusal does not reveal whether the email belongs to an account @credentialed</t>
         </is>
       </c>
       <c r="Q119" s="25" t="inlineStr">
@@ -15324,11 +15775,16 @@
       <c r="V119" s="15" t="n"/>
       <c r="W119" s="15" t="n"/>
       <c r="X119" s="15" t="n"/>
+      <c r="Y119" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-114</t>
+        </is>
+      </c>
     </row>
     <row r="120" ht="150" customHeight="1">
       <c r="A120" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-107</t>
+          <t>MS-ACC-001</t>
         </is>
       </c>
       <c r="B120" s="25" t="inlineStr">
@@ -15408,7 +15864,7 @@
       </c>
       <c r="P120" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-107 order history lists the member's orders with a number and a date each @smoke</t>
+          <t>MS-ACC-001 order history lists the member's orders with a number and a date each @smoke</t>
         </is>
       </c>
       <c r="Q120" s="25" t="inlineStr">
@@ -15433,11 +15889,16 @@
       <c r="V120" s="15" t="n"/>
       <c r="W120" s="15" t="n"/>
       <c r="X120" s="15" t="n"/>
+      <c r="Y120" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-107</t>
+        </is>
+      </c>
     </row>
     <row r="121" ht="150" customHeight="1">
       <c r="A121" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-108</t>
+          <t>MS-ACC-002</t>
         </is>
       </c>
       <c r="B121" s="25" t="inlineStr">
@@ -15516,7 +15977,7 @@
       </c>
       <c r="P121" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-108 selecting an order opens that order, not a placeholder</t>
+          <t>MS-ACC-002 selecting an order opens that order, not a placeholder</t>
         </is>
       </c>
       <c r="Q121" s="25" t="inlineStr">
@@ -15541,11 +16002,16 @@
       <c r="V121" s="15" t="n"/>
       <c r="W121" s="15" t="n"/>
       <c r="X121" s="15" t="n"/>
+      <c r="Y121" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-108</t>
+        </is>
+      </c>
     </row>
     <row r="122" ht="150" customHeight="1">
       <c r="A122" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-109</t>
+          <t>MS-ACC-003</t>
         </is>
       </c>
       <c r="B122" s="25" t="inlineStr">
@@ -15624,7 +16090,7 @@
       </c>
       <c r="P122" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-109 the 진행 중 / 이전 내역 control switches which orders are listed</t>
+          <t>MS-ACC-003 the 진행 중 / 이전 내역 control switches which orders are listed</t>
         </is>
       </c>
       <c r="Q122" s="25" t="inlineStr">
@@ -15649,11 +16115,16 @@
       <c r="V122" s="15" t="n"/>
       <c r="W122" s="15" t="n"/>
       <c r="X122" s="15" t="n"/>
+      <c r="Y122" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-109</t>
+        </is>
+      </c>
     </row>
     <row r="123" ht="150" customHeight="1">
       <c r="A123" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-110</t>
+          <t>MS-ACC-004</t>
         </is>
       </c>
       <c r="B123" s="25" t="inlineStr">
@@ -15732,7 +16203,7 @@
       </c>
       <c r="P123" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-110 order search narrows the list to the order that was searched for</t>
+          <t>MS-ACC-004 order search narrows the list to the order that was searched for</t>
         </is>
       </c>
       <c r="Q123" s="25" t="inlineStr">
@@ -15757,11 +16228,16 @@
       <c r="V123" s="15" t="n"/>
       <c r="W123" s="15" t="n"/>
       <c r="X123" s="15" t="n"/>
+      <c r="Y123" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-110</t>
+        </is>
+      </c>
     </row>
     <row r="124" ht="150" customHeight="1">
       <c r="A124" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-111</t>
+          <t>MS-ACC-005</t>
         </is>
       </c>
       <c r="B124" s="25" t="inlineStr">
@@ -15838,7 +16314,7 @@
       </c>
       <c r="P124" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-111 order history tools are present and named</t>
+          <t>MS-ACC-005 order history tools are present and named</t>
         </is>
       </c>
       <c r="Q124" s="25" t="inlineStr">
@@ -15863,11 +16339,16 @@
       <c r="V124" s="15" t="n"/>
       <c r="W124" s="15" t="n"/>
       <c r="X124" s="15" t="n"/>
+      <c r="Y124" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-111</t>
+        </is>
+      </c>
     </row>
     <row r="125" ht="150" customHeight="1">
       <c r="A125" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-017</t>
+          <t>MS-INQ-001</t>
         </is>
       </c>
       <c r="B125" s="25" t="inlineStr">
@@ -15945,7 +16426,7 @@
       </c>
       <c r="P125" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-017 inquiry form validates blank and invalid email submissions</t>
+          <t>MS-INQ-001 inquiry form validates blank and invalid email submissions</t>
         </is>
       </c>
       <c r="Q125" s="25" t="inlineStr">
@@ -15971,11 +16452,16 @@
       <c r="V125" s="15" t="n"/>
       <c r="W125" s="15" t="n"/>
       <c r="X125" s="15" t="n"/>
+      <c r="Y125" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-017</t>
+        </is>
+      </c>
     </row>
     <row r="126" ht="150" customHeight="1">
       <c r="A126" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-018</t>
+          <t>MS-INQ-002</t>
         </is>
       </c>
       <c r="B126" s="25" t="inlineStr">
@@ -16052,7 +16538,7 @@
       </c>
       <c r="P126" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-018 inquiry form documents supported attachment constraints</t>
+          <t>MS-INQ-002 inquiry form documents supported attachment constraints</t>
         </is>
       </c>
       <c r="Q126" s="25" t="inlineStr">
@@ -16078,11 +16564,16 @@
       <c r="V126" s="15" t="n"/>
       <c r="W126" s="15" t="n"/>
       <c r="X126" s="15" t="n"/>
+      <c r="Y126" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-018</t>
+        </is>
+      </c>
     </row>
     <row r="127" ht="150" customHeight="1">
       <c r="A127" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-019</t>
+          <t>MS-INQ-003</t>
         </is>
       </c>
       <c r="B127" s="25" t="inlineStr">
@@ -16159,7 +16650,7 @@
       </c>
       <c r="P127" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-019 external inquiry links point to Kakao and Naver destinations</t>
+          <t>MS-INQ-003 external inquiry links point to Kakao and Naver destinations</t>
         </is>
       </c>
       <c r="Q127" s="25" t="inlineStr">
@@ -16184,11 +16675,16 @@
       <c r="V127" s="15" t="n"/>
       <c r="W127" s="15" t="n"/>
       <c r="X127" s="15" t="n"/>
+      <c r="Y127" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-019</t>
+        </is>
+      </c>
     </row>
     <row r="128" ht="150" customHeight="1">
       <c r="A128" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-036</t>
+          <t>MS-API-001</t>
         </is>
       </c>
       <c r="B128" s="25" t="inlineStr">
@@ -16266,7 +16762,7 @@
       </c>
       <c r="P128" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-036 navigation categories API returns public category data</t>
+          <t>MS-API-001 navigation categories API returns public category data</t>
         </is>
       </c>
       <c r="Q128" s="25" t="inlineStr">
@@ -16291,11 +16787,16 @@
       <c r="V128" s="15" t="n"/>
       <c r="W128" s="15" t="n"/>
       <c r="X128" s="15" t="n"/>
+      <c r="Y128" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-036</t>
+        </is>
+      </c>
     </row>
     <row r="129" ht="150" customHeight="1">
       <c r="A129" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-037</t>
+          <t>MS-API-002</t>
         </is>
       </c>
       <c r="B129" s="25" t="inlineStr">
@@ -16373,7 +16874,7 @@
       </c>
       <c r="P129" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-037 inquiry types API returns selectable inquiry metadata</t>
+          <t>MS-API-002 inquiry types API returns selectable inquiry metadata</t>
         </is>
       </c>
       <c r="Q129" s="25" t="inlineStr">
@@ -16398,11 +16899,16 @@
       <c r="V129" s="15" t="n"/>
       <c r="W129" s="15" t="n"/>
       <c r="X129" s="15" t="n"/>
+      <c r="Y129" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-037</t>
+        </is>
+      </c>
     </row>
     <row r="130" ht="150" customHeight="1">
       <c r="A130" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-038</t>
+          <t>MS-API-003</t>
         </is>
       </c>
       <c r="B130" s="25" t="inlineStr">
@@ -16479,7 +16985,7 @@
       </c>
       <c r="P130" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-038 anonymous user session API rejects unauthenticated users safely</t>
+          <t>MS-API-003 anonymous user session API rejects unauthenticated users safely</t>
         </is>
       </c>
       <c r="Q130" s="25" t="inlineStr">
@@ -16504,11 +17010,16 @@
       <c r="V130" s="15" t="n"/>
       <c r="W130" s="15" t="n"/>
       <c r="X130" s="15" t="n"/>
+      <c r="Y130" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-038</t>
+        </is>
+      </c>
     </row>
     <row r="131" ht="150" customHeight="1">
       <c r="A131" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-023</t>
+          <t>MS-UX-001</t>
         </is>
       </c>
       <c r="B131" s="25" t="inlineStr">
@@ -16587,7 +17098,7 @@
       </c>
       <c r="P131" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-023 core controls are named and keyboard reachable</t>
+          <t>MS-UX-001 core controls are named and keyboard reachable</t>
         </is>
       </c>
       <c r="Q131" s="25" t="inlineStr">
@@ -16600,7 +17111,7 @@
       </c>
       <c r="S131" s="25" t="inlineStr">
         <is>
-          <t>Only one Tab press; focus is not checked to reach each control, and search is opened by mouse click, not Enter (test-case.md expects keyboard tabbing through all controls and Enter to open search). The header buttons are found by test id, so their accessible names are not verified here. The axe scan MS-V2-106 is the broader accessibility check.</t>
+          <t>Only one Tab press; focus is not checked to reach each control, and search is opened by mouse click, not Enter (test-case.md expects keyboard tabbing through all controls and Enter to open search). The header buttons are found by test id, so their accessible names are not verified here. The axe scan MS-UX-004 is the broader accessibility check.</t>
         </is>
       </c>
       <c r="T131" s="14" t="inlineStr">
@@ -16612,11 +17123,16 @@
       <c r="V131" s="15" t="n"/>
       <c r="W131" s="15" t="n"/>
       <c r="X131" s="15" t="n"/>
+      <c r="Y131" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-023</t>
+        </is>
+      </c>
     </row>
     <row r="132" ht="150" customHeight="1">
       <c r="A132" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-024</t>
+          <t>MS-UX-002</t>
         </is>
       </c>
       <c r="B132" s="25" t="inlineStr">
@@ -16695,7 +17211,7 @@
       </c>
       <c r="P132" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-024 home visual snapshot</t>
+          <t>MS-UX-002 home visual snapshot</t>
         </is>
       </c>
       <c r="Q132" s="25" t="inlineStr">
@@ -16720,11 +17236,16 @@
       <c r="V132" s="15" t="n"/>
       <c r="W132" s="15" t="n"/>
       <c r="X132" s="15" t="n"/>
+      <c r="Y132" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-024</t>
+        </is>
+      </c>
     </row>
     <row r="133" ht="150" customHeight="1">
       <c r="A133" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-043</t>
+          <t>MS-UX-003</t>
         </is>
       </c>
       <c r="B133" s="25" t="inlineStr">
@@ -16803,7 +17324,7 @@
       </c>
       <c r="P133" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-043 unknown route serves the 404 page with a working way back home</t>
+          <t>MS-UX-003 unknown route serves the 404 page with a working way back home</t>
         </is>
       </c>
       <c r="Q133" s="25" t="inlineStr">
@@ -16828,11 +17349,16 @@
       <c r="V133" s="15" t="n"/>
       <c r="W133" s="15" t="n"/>
       <c r="X133" s="15" t="n"/>
+      <c r="Y133" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-043</t>
+        </is>
+      </c>
     </row>
     <row r="134" ht="150" customHeight="1">
       <c r="A134" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-106</t>
+          <t>MS-UX-004</t>
         </is>
       </c>
       <c r="B134" s="25" t="inlineStr">
@@ -16911,7 +17437,7 @@
       </c>
       <c r="P134" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-106 home has no new WCAG AA violations</t>
+          <t>MS-UX-004 home has no new WCAG AA violations</t>
         </is>
       </c>
       <c r="Q134" s="25" t="inlineStr">
@@ -16936,6 +17462,11 @@
       <c r="V134" s="15" t="n"/>
       <c r="W134" s="15" t="n"/>
       <c r="X134" s="15" t="n"/>
+      <c r="Y134" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-106</t>
+        </is>
+      </c>
     </row>
     <row r="135" ht="150" customHeight="1">
       <c r="A135" s="12" t="inlineStr">
@@ -17679,7 +18210,7 @@
     <row r="142" ht="150" customHeight="1">
       <c r="A142" s="12" t="inlineStr">
         <is>
-          <t>MS-ADM-001</t>
+          <t>MS-ADMO-001</t>
         </is>
       </c>
       <c r="B142" s="25" t="inlineStr">
@@ -17765,7 +18296,7 @@
       </c>
       <c r="P142" s="25" t="inlineStr">
         <is>
-          <t>MS-ADM-001 artwork review, customer proof approval, production and delivery</t>
+          <t>MS-ADMO-001 artwork review, customer proof approval, production and delivery</t>
         </is>
       </c>
       <c r="Q142" s="25" t="inlineStr">
@@ -17802,11 +18333,16 @@
           <t>static-1. Every step has passed on the final code, but across two runs, not one uninterrupted run. Run 1 (AO-2609180003-dev) passed steps 1-7 and failed at step 8 on the redesigned approval dialog; with that fixed, the order was finished by a temporary script that found the other two flow changes (A-FPA label, no Move to Production). Run 2 (AO-2609090017-dev) with the updated spec passed steps 1-10 and failed at step 11 on the new no-results state of the order search; with that fixed, steps 11-12 passed against the same order. One seed order is left (AO-2609070006-dev) for a single clean run.</t>
         </is>
       </c>
+      <c r="Y142" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-ADM-001</t>
+        </is>
+      </c>
     </row>
     <row r="143" ht="150" customHeight="1">
       <c r="A143" s="12" t="inlineStr">
         <is>
-          <t>MS-ADM-007</t>
+          <t>MS-ADMO-002</t>
         </is>
       </c>
       <c r="B143" s="25" t="inlineStr">
@@ -17910,11 +18446,16 @@
       <c r="V143" s="15" t="n"/>
       <c r="W143" s="15" t="n"/>
       <c r="X143" s="15" t="n"/>
+      <c r="Y143" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-ADM-007</t>
+        </is>
+      </c>
     </row>
     <row r="144" ht="150" customHeight="1">
       <c r="A144" s="12" t="inlineStr">
         <is>
-          <t>MS-ADM-008</t>
+          <t>MS-ADMO-003</t>
         </is>
       </c>
       <c r="B144" s="25" t="inlineStr">
@@ -18017,11 +18558,16 @@
       <c r="V144" s="15" t="n"/>
       <c r="W144" s="15" t="n"/>
       <c r="X144" s="15" t="n"/>
+      <c r="Y144" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-ADM-008</t>
+        </is>
+      </c>
     </row>
     <row r="145" ht="150" customHeight="1">
       <c r="A145" s="12" t="inlineStr">
         <is>
-          <t>MS-ADM-009</t>
+          <t>MS-ADMO-004</t>
         </is>
       </c>
       <c r="B145" s="25" t="inlineStr">
@@ -18113,7 +18659,7 @@
       </c>
       <c r="S145" s="25" t="inlineStr">
         <is>
-          <t>Partly covered inside MS-ADM-001; this case isolates the rejection loop for quicker regression. Emails the member.</t>
+          <t>Partly covered inside MS-ADMO-001; this case isolates the rejection loop for quicker regression. Emails the member.</t>
         </is>
       </c>
       <c r="T145" s="14" t="inlineStr">
@@ -18125,11 +18671,16 @@
       <c r="V145" s="15" t="n"/>
       <c r="W145" s="15" t="n"/>
       <c r="X145" s="15" t="n"/>
+      <c r="Y145" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-ADM-009</t>
+        </is>
+      </c>
     </row>
     <row r="146" ht="150" customHeight="1">
       <c r="A146" s="12" t="inlineStr">
         <is>
-          <t>MS-ADM-010</t>
+          <t>MS-ADMO-005</t>
         </is>
       </c>
       <c r="B146" s="25" t="inlineStr">
@@ -18233,11 +18784,16 @@
       <c r="V146" s="15" t="n"/>
       <c r="W146" s="15" t="n"/>
       <c r="X146" s="15" t="n"/>
+      <c r="Y146" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-ADM-010</t>
+        </is>
+      </c>
     </row>
     <row r="147" ht="150" customHeight="1">
       <c r="A147" s="12" t="inlineStr">
         <is>
-          <t>MS-ADM-011</t>
+          <t>MS-ADMO-006</t>
         </is>
       </c>
       <c r="B147" s="25" t="inlineStr">
@@ -18340,11 +18896,16 @@
       <c r="V147" s="15" t="n"/>
       <c r="W147" s="15" t="n"/>
       <c r="X147" s="15" t="n"/>
+      <c r="Y147" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-ADM-011</t>
+        </is>
+      </c>
     </row>
     <row r="148" ht="150" customHeight="1">
       <c r="A148" s="12" t="inlineStr">
         <is>
-          <t>MS-ADM-012</t>
+          <t>MS-ADMO-007</t>
         </is>
       </c>
       <c r="B148" s="25" t="inlineStr">
@@ -18448,11 +19009,16 @@
       <c r="V148" s="15" t="n"/>
       <c r="W148" s="15" t="n"/>
       <c r="X148" s="15" t="n"/>
+      <c r="Y148" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-ADM-012</t>
+        </is>
+      </c>
     </row>
     <row r="149" ht="150" customHeight="1">
       <c r="A149" s="12" t="inlineStr">
         <is>
-          <t>MS-ADM-013</t>
+          <t>MS-ADMO-008</t>
         </is>
       </c>
       <c r="B149" s="25" t="inlineStr">
@@ -18555,11 +19121,16 @@
       <c r="V149" s="15" t="n"/>
       <c r="W149" s="15" t="n"/>
       <c r="X149" s="15" t="n"/>
+      <c r="Y149" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-ADM-013</t>
+        </is>
+      </c>
     </row>
     <row r="150" ht="150" customHeight="1">
       <c r="A150" s="12" t="inlineStr">
         <is>
-          <t>MS-ADM-014</t>
+          <t>MS-ADMO-009</t>
         </is>
       </c>
       <c r="B150" s="25" t="inlineStr">
@@ -18661,11 +19232,16 @@
       <c r="V150" s="15" t="n"/>
       <c r="W150" s="15" t="n"/>
       <c r="X150" s="15" t="n"/>
+      <c r="Y150" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-ADM-014</t>
+        </is>
+      </c>
     </row>
     <row r="151" ht="150" customHeight="1">
       <c r="A151" s="12" t="inlineStr">
         <is>
-          <t>MS-ADM-015</t>
+          <t>MS-ADMO-010</t>
         </is>
       </c>
       <c r="B151" s="25" t="inlineStr">
@@ -18756,7 +19332,7 @@
       </c>
       <c r="S151" s="25" t="inlineStr">
         <is>
-          <t>MUS-QA-004 fixed by 2026-10-14: the popup used to promise '제작 진행'; it now says 제작 대기, matching the behaviour. Covered end to end by MS-ADM-001 step 8. After approval the customer sees a cancellation notice citing a payment adjustment (MUS-QA-011).</t>
+          <t>MUS-QA-004 fixed by 2026-10-14: the popup used to promise '제작 진행'; it now says 제작 대기, matching the behaviour. Covered end to end by MS-ADMO-001 step 8. After approval the customer sees a cancellation notice citing a payment adjustment (MUS-QA-011).</t>
         </is>
       </c>
       <c r="T151" s="14" t="inlineStr">
@@ -18768,11 +19344,16 @@
       <c r="V151" s="15" t="n"/>
       <c r="W151" s="15" t="n"/>
       <c r="X151" s="15" t="n"/>
+      <c r="Y151" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-ADM-015</t>
+        </is>
+      </c>
     </row>
     <row r="152" ht="150" customHeight="1">
       <c r="A152" s="12" t="inlineStr">
         <is>
-          <t>MS-ADM-016</t>
+          <t>MS-ADMO-011</t>
         </is>
       </c>
       <c r="B152" s="25" t="inlineStr">
@@ -18863,7 +19444,7 @@
       </c>
       <c r="S152" s="25" t="inlineStr">
         <is>
-          <t>withdrawn 2026-10-14: Move to Production no longer exists on static-1. Mark as Printing (MS-ADM-017) is now the first staff action after approval and moves the order to 제작 진행 중 itself; the 주문 준비 중 (PO) stage is no longer reached. Keep the ID; do not reuse it.</t>
+          <t>withdrawn 2026-10-14: Move to Production no longer exists on static-1. Mark as Printing (MS-ADMO-012) is now the first staff action after approval and moves the order to 제작 진행 중 itself; the 주문 준비 중 (PO) stage is no longer reached. Keep the ID; do not reuse it.</t>
         </is>
       </c>
       <c r="T152" s="14" t="inlineStr">
@@ -18875,11 +19456,16 @@
       <c r="V152" s="15" t="n"/>
       <c r="W152" s="15" t="n"/>
       <c r="X152" s="15" t="n"/>
+      <c r="Y152" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-ADM-016</t>
+        </is>
+      </c>
     </row>
     <row r="153" ht="150" customHeight="1">
       <c r="A153" s="12" t="inlineStr">
         <is>
-          <t>MS-ADM-017</t>
+          <t>MS-ADMO-012</t>
         </is>
       </c>
       <c r="B153" s="25" t="inlineStr">
@@ -18982,11 +19568,16 @@
       <c r="V153" s="15" t="n"/>
       <c r="W153" s="15" t="n"/>
       <c r="X153" s="15" t="n"/>
+      <c r="Y153" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-ADM-017</t>
+        </is>
+      </c>
     </row>
     <row r="154" ht="150" customHeight="1">
       <c r="A154" s="12" t="inlineStr">
         <is>
-          <t>MS-ADM-018</t>
+          <t>MS-ADMO-013</t>
         </is>
       </c>
       <c r="B154" s="25" t="inlineStr">
@@ -19089,11 +19680,16 @@
       <c r="V154" s="15" t="n"/>
       <c r="W154" s="15" t="n"/>
       <c r="X154" s="15" t="n"/>
+      <c r="Y154" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-ADM-018</t>
+        </is>
+      </c>
     </row>
     <row r="155" ht="150" customHeight="1">
       <c r="A155" s="12" t="inlineStr">
         <is>
-          <t>MS-ADM-019</t>
+          <t>MS-ADMO-014</t>
         </is>
       </c>
       <c r="B155" s="25" t="inlineStr">
@@ -19195,11 +19791,16 @@
       <c r="V155" s="15" t="n"/>
       <c r="W155" s="15" t="n"/>
       <c r="X155" s="15" t="n"/>
+      <c r="Y155" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-ADM-019</t>
+        </is>
+      </c>
     </row>
     <row r="156" ht="150" customHeight="1">
       <c r="A156" s="12" t="inlineStr">
         <is>
-          <t>MS-ADM-020</t>
+          <t>MS-ADMO-015</t>
         </is>
       </c>
       <c r="B156" s="25" t="inlineStr">
@@ -19302,11 +19903,16 @@
       <c r="V156" s="15" t="n"/>
       <c r="W156" s="15" t="n"/>
       <c r="X156" s="15" t="n"/>
+      <c r="Y156" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-ADM-020</t>
+        </is>
+      </c>
     </row>
     <row r="157" ht="150" customHeight="1">
       <c r="A157" s="12" t="inlineStr">
         <is>
-          <t>MS-ADM-021</t>
+          <t>MS-ADMO-016</t>
         </is>
       </c>
       <c r="B157" s="25" t="inlineStr">
@@ -19407,11 +20013,16 @@
       <c r="V157" s="15" t="n"/>
       <c r="W157" s="15" t="n"/>
       <c r="X157" s="15" t="n"/>
+      <c r="Y157" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-ADM-021</t>
+        </is>
+      </c>
     </row>
     <row r="158" ht="150" customHeight="1">
       <c r="A158" s="12" t="inlineStr">
         <is>
-          <t>MS-ADM-025</t>
+          <t>MS-ADMO-017</t>
         </is>
       </c>
       <c r="B158" s="25" t="inlineStr">
@@ -19513,11 +20124,16 @@
       <c r="V158" s="15" t="n"/>
       <c r="W158" s="15" t="n"/>
       <c r="X158" s="15" t="n"/>
+      <c r="Y158" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-ADM-025</t>
+        </is>
+      </c>
     </row>
     <row r="159" ht="150" customHeight="1">
       <c r="A159" s="12" t="inlineStr">
         <is>
-          <t>MS-ADM-027</t>
+          <t>MS-ADMO-018</t>
         </is>
       </c>
       <c r="B159" s="25" t="inlineStr">
@@ -19619,11 +20235,16 @@
       <c r="V159" s="15" t="n"/>
       <c r="W159" s="15" t="n"/>
       <c r="X159" s="15" t="n"/>
+      <c r="Y159" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-ADM-027</t>
+        </is>
+      </c>
     </row>
     <row r="160" ht="150" customHeight="1">
       <c r="A160" s="12" t="inlineStr">
         <is>
-          <t>MS-ADM-002</t>
+          <t>MS-ADMA-001</t>
         </is>
       </c>
       <c r="B160" s="25" t="inlineStr">
@@ -19727,11 +20348,16 @@
       <c r="V160" s="15" t="n"/>
       <c r="W160" s="15" t="n"/>
       <c r="X160" s="15" t="n"/>
+      <c r="Y160" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-ADM-002</t>
+        </is>
+      </c>
     </row>
     <row r="161" ht="150" customHeight="1">
       <c r="A161" s="12" t="inlineStr">
         <is>
-          <t>MS-ADM-003</t>
+          <t>MS-ADMA-002</t>
         </is>
       </c>
       <c r="B161" s="25" t="inlineStr">
@@ -19836,11 +20462,16 @@
       <c r="V161" s="15" t="n"/>
       <c r="W161" s="15" t="n"/>
       <c r="X161" s="15" t="n"/>
+      <c r="Y161" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-ADM-003</t>
+        </is>
+      </c>
     </row>
     <row r="162" ht="150" customHeight="1">
       <c r="A162" s="12" t="inlineStr">
         <is>
-          <t>MS-ADM-004</t>
+          <t>MS-ADMA-003</t>
         </is>
       </c>
       <c r="B162" s="25" t="inlineStr">
@@ -19943,11 +20574,16 @@
       <c r="V162" s="15" t="n"/>
       <c r="W162" s="15" t="n"/>
       <c r="X162" s="15" t="n"/>
+      <c r="Y162" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-ADM-004</t>
+        </is>
+      </c>
     </row>
     <row r="163" ht="150" customHeight="1">
       <c r="A163" s="12" t="inlineStr">
         <is>
-          <t>MS-ADM-005</t>
+          <t>MS-ADMA-004</t>
         </is>
       </c>
       <c r="B163" s="25" t="inlineStr">
@@ -20052,11 +20688,16 @@
       <c r="V163" s="15" t="n"/>
       <c r="W163" s="15" t="n"/>
       <c r="X163" s="15" t="n"/>
+      <c r="Y163" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-ADM-005</t>
+        </is>
+      </c>
     </row>
     <row r="164" ht="150" customHeight="1">
       <c r="A164" s="12" t="inlineStr">
         <is>
-          <t>MS-ADM-006</t>
+          <t>MS-ADMA-005</t>
         </is>
       </c>
       <c r="B164" s="25" t="inlineStr">
@@ -20159,11 +20800,16 @@
       <c r="V164" s="15" t="n"/>
       <c r="W164" s="15" t="n"/>
       <c r="X164" s="15" t="n"/>
+      <c r="Y164" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-ADM-006</t>
+        </is>
+      </c>
     </row>
     <row r="165" ht="150" customHeight="1">
       <c r="A165" s="12" t="inlineStr">
         <is>
-          <t>MS-ADM-022</t>
+          <t>MS-ADMA-006</t>
         </is>
       </c>
       <c r="B165" s="25" t="inlineStr">
@@ -20198,7 +20844,7 @@
       </c>
       <c r="H165" s="25" t="inlineStr">
         <is>
-          <t>Admin panel static-1 (https://dev-static-1-admin-panel.musticker.com) signed in with a staff account. A test order taken through the lifecycle (e.g. after MS-ADM-001).</t>
+          <t>Admin panel static-1 (https://dev-static-1-admin-panel.musticker.com) signed in with a staff account. A test order taken through the lifecycle (e.g. after MS-ADMO-001).</t>
         </is>
       </c>
       <c r="I165" s="25" t="inlineStr">
@@ -20253,7 +20899,7 @@
       </c>
       <c r="S165" s="25" t="inlineStr">
         <is>
-          <t>Known defect 2026-09-25: the activity log records staff actions (Mark as Printing, tracking add/send/update; re-confirmed 2026-10-14) as the customer (user.is_admin=false). As of 2026-10-14 staff evaluation and proof entries (CA, FE, PE, NA) are correctly is_admin=true; printing and shipping entries (P, RS, OD, DE) are not. Audit-trail integrity issue; MS-ADM-001 deliberately asserts attribution only on customer steps until fixed.</t>
+          <t>Known defect 2026-09-25: the activity log records staff actions (Mark as Printing, tracking add/send/update; re-confirmed 2026-10-14) as the customer (user.is_admin=false). As of 2026-10-14 staff evaluation and proof entries (CA, FE, PE, NA) are correctly is_admin=true; printing and shipping entries (P, RS, OD, DE) are not. Audit-trail integrity issue; MS-ADMO-001 deliberately asserts attribution only on customer steps until fixed.</t>
         </is>
       </c>
       <c r="T165" s="14" t="inlineStr">
@@ -20265,11 +20911,16 @@
       <c r="V165" s="15" t="n"/>
       <c r="W165" s="15" t="n"/>
       <c r="X165" s="15" t="n"/>
+      <c r="Y165" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-ADM-022</t>
+        </is>
+      </c>
     </row>
     <row r="166" ht="150" customHeight="1">
       <c r="A166" s="12" t="inlineStr">
         <is>
-          <t>MS-ADM-023</t>
+          <t>MS-ADMA-007</t>
         </is>
       </c>
       <c r="B166" s="25" t="inlineStr">
@@ -20373,11 +21024,16 @@
       <c r="V166" s="15" t="n"/>
       <c r="W166" s="15" t="n"/>
       <c r="X166" s="15" t="n"/>
+      <c r="Y166" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-ADM-023</t>
+        </is>
+      </c>
     </row>
     <row r="167" ht="150" customHeight="1">
       <c r="A167" s="12" t="inlineStr">
         <is>
-          <t>MS-ADM-024</t>
+          <t>MS-ADMA-008</t>
         </is>
       </c>
       <c r="B167" s="25" t="inlineStr">
@@ -20479,11 +21135,16 @@
       <c r="V167" s="15" t="n"/>
       <c r="W167" s="15" t="n"/>
       <c r="X167" s="15" t="n"/>
+      <c r="Y167" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-ADM-024</t>
+        </is>
+      </c>
     </row>
     <row r="168" ht="150" customHeight="1">
       <c r="A168" s="12" t="inlineStr">
         <is>
-          <t>MS-ADM-026</t>
+          <t>MS-ADMA-009</t>
         </is>
       </c>
       <c r="B168" s="25" t="inlineStr">
@@ -20586,11 +21247,16 @@
       <c r="V168" s="15" t="n"/>
       <c r="W168" s="15" t="n"/>
       <c r="X168" s="15" t="n"/>
+      <c r="Y168" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-ADM-026</t>
+        </is>
+      </c>
     </row>
     <row r="169" ht="150" customHeight="1">
       <c r="A169" s="12" t="inlineStr">
         <is>
-          <t>MS-ADM-028</t>
+          <t>MS-ADMA-010</t>
         </is>
       </c>
       <c r="B169" s="25" t="inlineStr">
@@ -20688,11 +21354,16 @@
       <c r="V169" s="15" t="n"/>
       <c r="W169" s="15" t="n"/>
       <c r="X169" s="15" t="n"/>
+      <c r="Y169" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-ADM-028</t>
+        </is>
+      </c>
     </row>
     <row r="170" ht="150" customHeight="1">
       <c r="A170" s="12" t="inlineStr">
         <is>
-          <t>MS-ADM-029</t>
+          <t>MS-ADMA-011</t>
         </is>
       </c>
       <c r="B170" s="25" t="inlineStr">
@@ -20795,11 +21466,16 @@
       <c r="V170" s="15" t="n"/>
       <c r="W170" s="15" t="n"/>
       <c r="X170" s="15" t="n"/>
+      <c r="Y170" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-ADM-029</t>
+        </is>
+      </c>
     </row>
     <row r="171" ht="150" customHeight="1">
       <c r="A171" s="12" t="inlineStr">
         <is>
-          <t>MS-ADM-030</t>
+          <t>MS-ADMA-012</t>
         </is>
       </c>
       <c r="B171" s="25" t="inlineStr">
@@ -20901,11 +21577,16 @@
       <c r="V171" s="15" t="n"/>
       <c r="W171" s="15" t="n"/>
       <c r="X171" s="15" t="n"/>
+      <c r="Y171" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-ADM-030</t>
+        </is>
+      </c>
     </row>
     <row r="172" ht="150" customHeight="1">
       <c r="A172" s="12" t="inlineStr">
         <is>
-          <t>MS-ADM-031</t>
+          <t>MS-ADMA-013</t>
         </is>
       </c>
       <c r="B172" s="25" t="inlineStr">
@@ -20940,7 +21621,7 @@
       </c>
       <c r="H172" s="25" t="inlineStr">
         <is>
-          <t>Seeded member signed in on static-1 storefront; a test order at 주문 완료 (e.g. after MS-ADM-001).</t>
+          <t>Seeded member signed in on static-1 storefront; a test order at 주문 완료 (e.g. after MS-ADMO-001).</t>
         </is>
       </c>
       <c r="I172" s="25" t="inlineStr">
@@ -21007,11 +21688,16 @@
       <c r="V172" s="15" t="n"/>
       <c r="W172" s="15" t="n"/>
       <c r="X172" s="15" t="n"/>
+      <c r="Y172" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-ADM-031</t>
+        </is>
+      </c>
     </row>
     <row r="173" ht="150" customHeight="1">
       <c r="A173" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-115</t>
+          <t>MS-CFG-026</t>
         </is>
       </c>
       <c r="B173" s="25" t="inlineStr">
@@ -21088,7 +21774,7 @@
       </c>
       <c r="P173" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-115 다음 단계 offers three ways to order: with a file, in the studio, or file later</t>
+          <t>MS-CFG-026 다음 단계 offers three ways to order: with a file, in the studio, or file later</t>
         </is>
       </c>
       <c r="Q173" s="25" t="inlineStr">
@@ -21113,11 +21799,16 @@
       <c r="V173" s="15" t="n"/>
       <c r="W173" s="15" t="n"/>
       <c r="X173" s="15" t="n"/>
+      <c r="Y173" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-115</t>
+        </is>
+      </c>
     </row>
     <row r="174" ht="150" customHeight="1">
       <c r="A174" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-116</t>
+          <t>MS-CFG-027</t>
         </is>
       </c>
       <c r="B174" s="25" t="inlineStr">
@@ -21196,7 +21887,7 @@
       </c>
       <c r="P174" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-116 the studio keeps the configured size and quantity and prices every tier 5% below the configurator</t>
+          <t>MS-CFG-027 the studio keeps the configured size and quantity and prices every tier 5% below the configurator</t>
         </is>
       </c>
       <c r="Q174" s="25" t="inlineStr">
@@ -21221,11 +21912,16 @@
       <c r="V174" s="15" t="n"/>
       <c r="W174" s="15" t="n"/>
       <c r="X174" s="15" t="n"/>
+      <c r="Y174" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-116</t>
+        </is>
+      </c>
     </row>
     <row r="175" ht="150" customHeight="1">
       <c r="A175" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-117</t>
+          <t>MS-CFG-028</t>
         </is>
       </c>
       <c r="B175" s="25" t="inlineStr">
@@ -21270,7 +21966,7 @@
       </c>
       <c r="J175" s="25" t="inlineStr">
         <is>
-          <t>1. Open the studio for 자유형 조각스티커 at 중형 75x75 / 100개 (as MS-V2-116).
+          <t>1. Open the studio for 자유형 조각스티커 at 중형 75x75 / 100개 (as MS-CFG-027).
 2. Check 장바구니 담기 before attaching anything.
 3. Click 이미지 첨부하기 and choose qa-proof.png.
 4. Open a fresh studio the same way and attach studio-design.png.</t>
@@ -21303,7 +21999,7 @@
       </c>
       <c r="P175" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-117 the studio refuses a low-resolution design and accepts a print-quality one</t>
+          <t>MS-CFG-028 the studio refuses a low-resolution design and accepts a print-quality one</t>
         </is>
       </c>
       <c r="Q175" s="25" t="inlineStr">
@@ -21328,11 +22024,16 @@
       <c r="V175" s="15" t="n"/>
       <c r="W175" s="15" t="n"/>
       <c r="X175" s="15" t="n"/>
+      <c r="Y175" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-117</t>
+        </is>
+      </c>
     </row>
     <row r="176" ht="150" customHeight="1">
       <c r="A176" s="12" t="inlineStr">
         <is>
-          <t>MS-V2-118</t>
+          <t>MS-CFG-029</t>
         </is>
       </c>
       <c r="B176" s="25" t="inlineStr">
@@ -21377,7 +22078,7 @@
       </c>
       <c r="J176" s="25" t="inlineStr">
         <is>
-          <t>1. Open the studio with a print-quality design attached (MS-V2-117 step 4).
+          <t>1. Open the studio with a print-quality design attached (MS-CFG-028 step 4).
 2. Click 장바구니 담기.
 3. In 주문 준비 완료, wait for the preview, look through the 미리보기 대상 scenes, choose 재단 방식 (통재단 / 도무송).
 4. Tick 네, 확인했어요! and click 장바구니 담기.
@@ -21436,9 +22137,14 @@
       <c r="V176" s="15" t="n"/>
       <c r="W176" s="15" t="n"/>
       <c r="X176" s="15" t="n"/>
+      <c r="Y176" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS-V2-118</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:X176"/>
+  <autoFilter ref="A1:Y176"/>
   <dataValidations count="3">
     <dataValidation sqref="T2:T176" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Not Run,Pass,Fail,Blocked,Partial,N/A"</formula1>
@@ -21705,7 +22411,7 @@
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
         <is>
-          <t>ADMIN SEED ORDERS (MS-ADM-001, static-1)</t>
+          <t>ADMIN SEED ORDERS (MS-ADMO-001, static-1)</t>
         </is>
       </c>
       <c r="B14" s="8" t="n"/>
@@ -21769,12 +22475,12 @@
       </c>
       <c r="C17" s="25" t="inlineStr">
         <is>
-          <t>exploration 2026-09-25; MS-ADM-001 2026-10-14; other testers</t>
+          <t>exploration 2026-09-25; MS-ADMO-001 2026-10-14; other testers</t>
         </is>
       </c>
       <c r="D17" s="25" t="inlineStr">
         <is>
-          <t>AO-2609240008/2609250005: walked by hand 2026-09-25. AO-2609180003/2609090017: MS-ADM-001 runs 2026-10-14. AO-2609180004: found at 승인 대기 on 2026-10-14 (used by someone else). Not usable: AO-2609070004-dev and AO-2609070005-dev have two items each.</t>
+          <t>AO-2609240008/2609250005: walked by hand 2026-09-25. AO-2609180003/2609090017: MS-ADMO-001 runs 2026-10-14. AO-2609180004: found at 승인 대기 on 2026-10-14 (used by someone else). Not usable: AO-2609070004-dev and AO-2609070005-dev have two items each.</t>
         </is>
       </c>
     </row>
@@ -21828,7 +22534,7 @@
       </c>
       <c r="D20" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-098 / 099.</t>
+          <t>MS-CHK-005 / MS-CHK-006.</t>
         </is>
       </c>
     </row>
@@ -22007,7 +22713,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Verified by hand on static-1 (dev-static-1) on 2026-09-25 (AO-2609240008-dev, AO-2609250005-dev) and re-checked by MS-ADM-001 on 2026-10-14 (AO-2609180003-dev, AO-2609090017-dev). The reference when a case and the product disagree.</t>
+          <t>Verified by hand on static-1 (dev-static-1) on 2026-09-25 (AO-2609240008-dev, AO-2609250005-dev) and re-checked by MS-ADMO-001 on 2026-10-14 (AO-2609180003-dev, AO-2609090017-dev). The reference when a case and the product disagree.</t>
         </is>
       </c>
     </row>
@@ -24670,7 +25376,7 @@
       </c>
       <c r="C2" s="25" t="inlineStr">
         <is>
-          <t>MS-ADM-022</t>
+          <t>MS-ADMA-006</t>
         </is>
       </c>
       <c r="D2" s="25" t="inlineStr">
@@ -24755,7 +25461,7 @@
       </c>
       <c r="C3" s="25" t="inlineStr">
         <is>
-          <t>MS-ADM-024</t>
+          <t>MS-ADMA-008</t>
         </is>
       </c>
       <c r="D3" s="25" t="inlineStr">
@@ -24840,7 +25546,7 @@
       </c>
       <c r="C4" s="25" t="inlineStr">
         <is>
-          <t>MS-ADM-021</t>
+          <t>MS-ADMO-016</t>
         </is>
       </c>
       <c r="D4" s="25" t="inlineStr">
@@ -24925,7 +25631,7 @@
       </c>
       <c r="C5" s="25" t="inlineStr">
         <is>
-          <t>MS-ADM-015</t>
+          <t>MS-ADMO-010</t>
         </is>
       </c>
       <c r="D5" s="25" t="inlineStr">
@@ -25016,7 +25722,7 @@
       </c>
       <c r="C6" s="25" t="inlineStr">
         <is>
-          <t>MS-ADM-008</t>
+          <t>MS-ADMO-003</t>
         </is>
       </c>
       <c r="D6" s="25" t="inlineStr">
@@ -25102,7 +25808,7 @@
       </c>
       <c r="C7" s="25" t="inlineStr">
         <is>
-          <t>MS-ADM-030</t>
+          <t>MS-ADMA-012</t>
         </is>
       </c>
       <c r="D7" s="25" t="inlineStr">
@@ -25187,7 +25893,7 @@
       </c>
       <c r="C8" s="25" t="inlineStr">
         <is>
-          <t>MS-ADM-031</t>
+          <t>MS-ADMA-013</t>
         </is>
       </c>
       <c r="D8" s="25" t="inlineStr">
@@ -25276,7 +25982,7 @@
       </c>
       <c r="C9" s="25" t="inlineStr">
         <is>
-          <t>MS-ADM-007</t>
+          <t>MS-ADMO-002</t>
         </is>
       </c>
       <c r="D9" s="25" t="inlineStr">
@@ -25361,7 +26067,7 @@
       </c>
       <c r="C10" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-109</t>
+          <t>MS-ACC-003</t>
         </is>
       </c>
       <c r="D10" s="25" t="inlineStr">
@@ -25446,7 +26152,7 @@
       </c>
       <c r="C11" s="25" t="inlineStr">
         <is>
-          <t>MS-ADM-020</t>
+          <t>MS-ADMO-015</t>
         </is>
       </c>
       <c r="D11" s="25" t="inlineStr">
@@ -25502,7 +26208,7 @@
       </c>
       <c r="N11" s="25" t="inlineStr">
         <is>
-          <t>MS-ADM-001 run (automation)</t>
+          <t>MS-ADMO-001 run (automation)</t>
         </is>
       </c>
       <c r="O11" s="25" t="inlineStr">
@@ -25531,7 +26237,7 @@
       </c>
       <c r="C12" s="25" t="inlineStr">
         <is>
-          <t>MS-ADM-015</t>
+          <t>MS-ADMO-010</t>
         </is>
       </c>
       <c r="D12" s="25" t="inlineStr">
@@ -25587,7 +26293,7 @@
       </c>
       <c r="N12" s="25" t="inlineStr">
         <is>
-          <t>MS-ADM-001 run (automation)</t>
+          <t>MS-ADMO-001 run (automation)</t>
         </is>
       </c>
       <c r="O12" s="25" t="inlineStr">
@@ -25616,7 +26322,7 @@
       </c>
       <c r="C13" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-003</t>
+          <t>MS-NAV-003</t>
         </is>
       </c>
       <c r="D13" s="25" t="inlineStr">
@@ -25701,7 +26407,7 @@
       </c>
       <c r="C14" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-009</t>
+          <t>MS-CFG-001</t>
         </is>
       </c>
       <c r="D14" s="25" t="inlineStr">
@@ -25786,7 +26492,7 @@
       </c>
       <c r="C15" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-009</t>
+          <t>MS-CFG-001</t>
         </is>
       </c>
       <c r="D15" s="25" t="inlineStr">
@@ -25871,7 +26577,7 @@
       </c>
       <c r="C16" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-118</t>
+          <t>MS-CFG-029</t>
         </is>
       </c>
       <c r="D16" s="25" t="inlineStr">
@@ -25956,7 +26662,7 @@
       </c>
       <c r="C17" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-002</t>
+          <t>MS-NAV-002</t>
         </is>
       </c>
       <c r="D17" s="25" t="inlineStr">
@@ -26041,7 +26747,7 @@
       </c>
       <c r="C18" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-009</t>
+          <t>MS-CFG-001</t>
         </is>
       </c>
       <c r="D18" s="25" t="inlineStr">
@@ -26126,7 +26832,7 @@
       </c>
       <c r="C19" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-116</t>
+          <t>MS-CFG-027</t>
         </is>
       </c>
       <c r="D19" s="25" t="inlineStr">
@@ -26211,7 +26917,7 @@
       </c>
       <c r="C20" s="25" t="inlineStr">
         <is>
-          <t>MS-V2-106</t>
+          <t>MS-UX-004</t>
         </is>
       </c>
       <c r="D20" s="25" t="inlineStr">
@@ -26372,7 +27078,7 @@
     <row r="23">
       <c r="A23" s="24" t="inlineStr">
         <is>
-          <t>MUS-QA-001 to 009 were found by exploratory testing on 2026-09-25 while building the admin suite, MUS-QA-010 and 011 by the MS-ADM-001 run on 2026-10-14, and MUS-QA-012 to 020 by storefront exploration the same day. Evidence gives order numbers and times so dev can find the records. Add new defects below; keep IDs sequential.</t>
+          <t>MUS-QA-001 to 009 were found by exploratory testing on 2026-09-25 while building the admin suite, MUS-QA-010 and 011 by the MS-ADMO-001 run on 2026-10-14, and MUS-QA-012 to 020 by storefront exploration the same day. Evidence gives order numbers and times so dev can find the records. Add new defects below; keep IDs sequential.</t>
         </is>
       </c>
     </row>
@@ -26402,7 +27108,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B34"/>
+  <dimension ref="A1:B39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -26426,299 +27132,298 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>2026-10-14 - workbook v1.1, MS-ADM-001 re-run, storefront explored</t>
+          <t xml:space="preserve">2026-10-14 - workbook v1.2, module-based TC IDs</t>
         </is>
       </c>
     </row>
     <row r="5" ht="38.25" customHeight="1">
       <c r="A5" s="28" t="inlineStr">
         <is>
-          <t>MS-ADM-001</t>
+          <t xml:space="preserve">TC IDs</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Re-run on static-1 (AO-2609180003-dev, AO-2609090017-dev) and updated for four product changes: the proof-approval dialog needs an acknowledgement tick before 최종 시안 승인; A-FPA is labelled 최종 승인 완료; Move to Production is gone, so Mark as Printing moves the order to 제작 진행 중 and the item straight to 인쇄 진행 중 (no PO); completed orders moved to 이전 내역, and an order search with no match shows 주문을 찾을 수 없습니다. Every step passes on the updated code (see Tester Notes on the case).</t>
+          <t xml:space="preserve">MS-V2-### and MS-ADM-### are replaced by MS-&lt;MODULE&gt;-###, so an ID names its module (the Area): NAV, DSC, CFG, SHT, CRT, CHK, AUTH, ACC, INQ, API, UX, ADMO (admin order processing) and ADMA (admin access &amp; order management), numbered 001 upward in workbook order. MS-PRC-*, MS-SEC-* and MS-WAF-* are unchanged. 140 cases renamed.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="38.25" customHeight="1">
       <c r="A6" s="28" t="inlineStr">
         <is>
+          <t xml:space="preserve">Legacy ID</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">New column Y keeps each renamed case's previous ID. Older entries in this changelog, past Allure history and defect evidence still use the old IDs; look them up in that column.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="38.25" customHeight="1">
+      <c r="A7" s="28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Suite</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Playwright test titles, comments, fixtures and docs renamed to match (178 test titles; no test logic changed; still 2,473 tests). Defect Log TC IDs and the cross-references in the other tabs updated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-14 - workbook v1.1, MS-ADM-001 re-run, storefront explored</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="38.25" customHeight="1">
+      <c r="A10" s="28" t="inlineStr">
+        <is>
+          <t>MS-ADM-001</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Re-run on static-1 (AO-2609180003-dev, AO-2609090017-dev) and updated for four product changes: the proof-approval dialog needs an acknowledgement tick before 최종 시안 승인; A-FPA is labelled 최종 승인 완료; Move to Production is gone, so Mark as Printing moves the order to 제작 진행 중 and the item straight to 인쇄 진행 중 (no PO); completed orders moved to 이전 내역, and an order search with no match shows 주문을 찾을 수 없습니다. Every step passes on the updated code (see Tester Notes on the case).</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="38.25" customHeight="1">
+      <c r="A11" s="28" t="inlineStr">
+        <is>
           <t>Admin recording</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B11" s="5" t="inlineStr">
         <is>
           <t>A failed run showed that Playwright's failure screenshot and error context capture every open page, the admin panel included - the suite promised they did not. Admin specs now turn screenshots and traces off, and the adminPage fixture refuses to start otherwise.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="25.5" customHeight="1">
-      <c r="A7" s="28" t="inlineStr">
-        <is>
-          <t>Cases</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>MS-ADM-016 (Move to Production) withdrawn. MS-ADM-006, 013, 014, 015, 017, 020, 022, 030 and 031 updated to the new flow; Business Rules and Glossary likewise.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="28" t="inlineStr">
-        <is>
-          <t>Defects</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>MUS-QA-004 and MUS-QA-007 retested as fixed. MUS-QA-001 still reproduces for the printing and shipping entries. New: MUS-QA-010 and MUS-QA-011 (Low, to confirm).</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="28" t="inlineStr">
-        <is>
-          <t>Environments</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>Instructions, gating, the Test Plan, Test Data and pricing ids now use the current environment names (static-1..8; development-1..4 retired and development-static/-static-2 renamed on 2026-09-25), and the CI schedule no longer lists the removed nightly regression. Historical "verified on development-N" notes are kept as they were.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="28" t="inlineStr">
-        <is>
-          <t>Seed orders</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>Re-checked on 2026-10-14: AO-2609180004-dev had been used elsewhere and AO-2609070004/0005-dev have two items, so one unused candidate is left (AO-2609070006-dev).</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="28" t="inlineStr">
-        <is>
-          <t>Admin login</t>
-        </is>
-      </c>
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>dev-static-1 has a tester OTP endpoint that returns the admin verification code; noted under MS-ADM-002 as a way to run admin cases without a person. Not used by the suite yet.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="25.5" customHeight="1">
       <c r="A12" s="28" t="inlineStr">
         <is>
-          <t>Storefront run</t>
+          <t>Cases</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Production-safe storefront specs (pricing excluded) before the updates: production 132 passed / 27 failed / 5 flaky; static-1 131 / 28 / 5. After: production 162 passed, 2 failed and 3 flaky (a tier-price repaint race, fixed and then 32/32 twice; transient 502s), 5 skipped; static-1 165 passed, 0 failed, 2 flaky (a network blip; MS-V2-035's timeout, now 90 s and passing on both), 5 skipped. Pricing on production: 261 of 2,286 failed, all on the replaced lettering and transfer tables; after the re-export 272/272 for those two and the other 2,016 unchanged and passing.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="25.5" customHeight="1">
+          <t>MS-ADM-016 (Move to Production) withdrawn. MS-ADM-006, 013, 014, 015, 017, 020, 022, 030 and 031 updated to the new flow; Business Rules and Glossary likewise.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
       <c r="A13" s="28" t="inlineStr">
         <is>
-          <t>Order chooser</t>
+          <t>Defects</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>다음 단계 now opens 어떻게 주문하시겠어요? (with a file / in the studio / file later), live on production. MS-V2-050 and 053 updated; new MS-V2-115.</t>
+          <t>MUS-QA-004 and MUS-QA-007 retested as fixed. MUS-QA-001 still reproduces for the printing and shipping entries. New: MUS-QA-010 and MUS-QA-011 (Low, to confirm).</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="28" t="inlineStr">
         <is>
-          <t>Design studio</t>
+          <t>Environments</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>New web studio (?studio=1): carries size and quantity over, prices 5% lower, refuses low-resolution designs. New MS-V2-116 and 117 (automated, production-safe) and MS-V2-118 (planned: add-to-cart blocked by MUS-QA-015). New fixture studio-design.png.</t>
+          <t>Instructions, gating, the Test Plan, Test Data and pricing ids now use the current environment names (static-1..8; development-1..4 retired and development-static/-static-2 renamed on 2026-09-25), and the CI schedule no longer lists the removed nightly regression. Historical "verified on development-N" notes are kept as they were.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="28" t="inlineStr">
         <is>
-          <t>Header and footer</t>
+          <t>Seed orders</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>Nav items open a product menu instead of the category page (MS-V2-002 rewritten, MS-V2-035 updated); the footer was redesigned (MS-V2-001, 020, 039).</t>
+          <t>Re-checked on 2026-10-14: AO-2609180004-dev had been used elsewhere and AO-2609070004/0005-dev have two items, so one unused candidate is left (AO-2609070006-dev).</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="28" t="inlineStr">
         <is>
-          <t>Copy and options</t>
+          <t>Admin login</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>PVC 매트 is now 무광 화이트; sheet stickers show a discount on every tier (MS-V2-052 rewritten); rounded-roll, rounded-sheet and transfer H1s renamed back; production's category cards reverted to pre-rename names (MUS-QA-016).</t>
+          <t>dev-static-1 has a tester OTP endpoint that returns the admin verification code; noted under MS-ADM-002 as a way to run admin cases without a person. Not used by the suite yet.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="25.5" customHeight="1">
       <c r="A17" s="28" t="inlineStr">
         <is>
-          <t>Suite fixes</t>
+          <t>Storefront run</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>selectSize waits for the size re-quote (stale tier prices failed the money-path tests); quantity tiers match the whole number (5 had been picking 50시트); category menu and review carousel clicks wait for Nuxt hydration (new waitForNuxtHydration); addToCart handles both the chooser and the older upload dialog (풀 컬러 레터링); the unused-preload warning is benign on every first-party host; new allowStudioModelLoadNoise guard option.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
+          <t>Production-safe storefront specs (pricing excluded) before the updates: production 132 passed / 27 failed / 5 flaky; static-1 131 / 28 / 5. After: production 162 passed, 2 failed and 3 flaky (a tier-price repaint race, fixed and then 32/32 twice; transient 502s), 5 skipped; static-1 165 passed, 0 failed, 2 flaky (a network blip; MS-V2-035's timeout, now 90 s and passing on both), 5 skipped. Pricing on production: 261 of 2,286 failed, all on the replaced lettering and transfer tables; after the re-export 272/272 for those two and the other 2,016 unchanged and passing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="25.5" customHeight="1">
       <c r="A18" s="28" t="inlineStr">
         <is>
-          <t>Pricing</t>
+          <t>Order chooser</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>Production replaced the vinyl-lettering and transfer-sticker tables on 2026-09-29 (ids 69 and 72; same rates on rungs 1-300, new rungs 500-5,000): CSVs re-exported, registry updated, now production-only baselines. The known interpolation overcharge checks are pinned to their quantities (the longer ladder had moved the sampled quantity off them and hidden that the overcharge is still live). Pricing now 2,288 tests.</t>
+          <t>다음 단계 now opens 어떻게 주문하시겠어요? (with a file / in the studio / file later), live on production. MS-V2-050 and 053 updated; new MS-V2-115.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="28" t="inlineStr">
         <is>
+          <t>Design studio</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>New web studio (?studio=1): carries size and quantity over, prices 5% lower, refuses low-resolution designs. New MS-V2-116 and 117 (automated, production-safe) and MS-V2-118 (planned: add-to-cart blocked by MUS-QA-015). New fixture studio-design.png.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="28" t="inlineStr">
+        <is>
+          <t>Header and footer</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Nav items open a product menu instead of the category page (MS-V2-002 rewritten, MS-V2-035 updated); the footer was redesigned (MS-V2-001, 020, 039).</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="28" t="inlineStr">
+        <is>
+          <t>Copy and options</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>PVC 매트 is now 무광 화이트; sheet stickers show a discount on every tier (MS-V2-052 rewritten); rounded-roll, rounded-sheet and transfer H1s renamed back; production's category cards reverted to pre-rename names (MUS-QA-016).</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="25.5" customHeight="1">
+      <c r="A22" s="28" t="inlineStr">
+        <is>
+          <t>Suite fixes</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>selectSize waits for the size re-quote (stale tier prices failed the money-path tests); quantity tiers match the whole number (5 had been picking 50시트); category menu and review carousel clicks wait for Nuxt hydration (new waitForNuxtHydration); addToCart handles both the chooser and the older upload dialog (풀 컬러 레터링); the unused-preload warning is benign on every first-party host; new allowStudioModelLoadNoise guard option.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="28" t="inlineStr">
+        <is>
+          <t>Pricing</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>Production replaced the vinyl-lettering and transfer-sticker tables on 2026-09-29 (ids 69 and 72; same rates on rungs 1-300, new rungs 500-5,000): CSVs re-exported, registry updated, now production-only baselines. The known interpolation overcharge checks are pinned to their quantities (the longer ladder had moved the sampled quantity off them and hidden that the overcharge is still live). Pricing now 2,288 tests.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="28" t="inlineStr">
+        <is>
           <t>Storefront defects</t>
         </is>
       </c>
-      <c r="B19" s="5" t="inlineStr">
+      <c r="B24" s="5" t="inlineStr">
         <is>
           <t>MUS-QA-012 to 020 logged (search button name, /dev/ assets on production, page weight, studio confirmation lock, pre-rename names, English FAQ on static-1, size-range mismatch, selection state not exposed, lettering 500-rung rate).</t>
         </is>
       </c>
     </row>
-    <row r="20"/>
-    <row r="21">
-      <c r="A21" s="3" t="inlineStr">
+    <row r="25"/>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
         <is>
           <t>2026-09-25 - workbook v1, suite reorganised</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="4" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
         <is>
           <t>Workbook</t>
         </is>
       </c>
-      <c r="B22" s="5" t="inlineStr">
+      <c r="B27" s="5" t="inlineStr">
         <is>
           <t>This workbook replaces test-case.md as the test case source. Steps and expected results were re-derived from the spec code (the code is the source of truth); where test-case.md described more than the code checks, the case says so in Reference Notes, and three cases are marked Partial (MS-V2-012, 017, 018).</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="4" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
         <is>
           <t>Admin panel</t>
         </is>
       </c>
-      <c r="B23" s="5" t="inlineStr">
+      <c r="B28" s="5" t="inlineStr">
         <is>
           <t>Added the admin panel to the suite: MS-ADM-001 (storefront-to-admin order processing: design upload, rejection and resubmission, pass, proof, customer approval, production, printing, shipping, delivery) plus planned admin cases (MS-ADM-002 onward).</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="4" t="inlineStr">
-        <is>
-          <t>Folders</t>
-        </is>
-      </c>
-      <c r="B24" s="5" t="inlineStr">
-        <is>
-          <t>Specs moved to tests/e2e/storefront/&lt;area&gt;/ and tests/e2e/admin/&lt;area&gt;/; page objects to tests/pom/storefront/ and tests/pom/admin/. Same 2,468 tests before and after (verified by comparing the test lists).</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="4" t="inlineStr">
-        <is>
-          <t>Docs</t>
-        </is>
-      </c>
-      <c r="B25" s="5" t="inlineStr">
-        <is>
-          <t>New docs/RUNNING.md, docs/ARCHITECTURE.md, docs/CONVENTIONS.md; README.md is now a short entry point.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="4" t="inlineStr">
-        <is>
-          <t>Defects</t>
-        </is>
-      </c>
-      <c r="B26" s="5" t="inlineStr">
-        <is>
-          <t>Nine defects/questions from exploratory testing logged (MUS-QA-001 to 009).</t>
-        </is>
-      </c>
-    </row>
-    <row r="27"/>
-    <row r="28">
-      <c r="A28" s="3" t="inlineStr">
-        <is>
-          <t>KNOWN SUITE ISSUES (not product defects)</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>dev-static-1 checkout</t>
+          <t>Folders</t>
         </is>
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>Cloudflare check before payment blocks automated browsers; guest checkout there shows no OTP popup on email blur. MS-V2-025 is verified on development-3 only.</t>
+          <t>Specs moved to tests/e2e/storefront/&lt;area&gt;/ and tests/e2e/admin/&lt;area&gt;/; page objects to tests/pom/storefront/ and tests/pom/admin/. Same 2,468 tests before and after (verified by comparing the test lists).</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>Upload dialog (dev-static-1)</t>
+          <t>Docs</t>
         </is>
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>The product upload dialog button is now 파일로 주문하기 and the file-type copy reads 'ai · psd · pdf · eps · tif · png · jpg'. ProductV2Page.expectDesignUploadModal and MS-V2-053 will fail when this reaches production - update storefront-data.ts then.</t>
+          <t>New docs/RUNNING.md, docs/ARCHITECTURE.md, docs/CONVENTIONS.md; README.md is now a short entry point.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>MS-V2-058</t>
+          <t>Defects</t>
         </is>
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>Marked test.fixme (known alt-text defect on the size guide); skipped until fixed.</t>
+          <t>Nine defects/questions from exploratory testing logged (MUS-QA-001 to 009).</t>
         </is>
       </c>
     </row>
@@ -26726,17 +27431,61 @@
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>2026-08-10 - test-case.md v1</t>
+          <t>KNOWN SUITE ISSUES (not product defects)</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
         <is>
+          <t>dev-static-1 checkout</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>Cloudflare check before payment blocks automated browsers; guest checkout there shows no OTP popup on email blur. MS-V2-025 is verified on development-3 only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Upload dialog (dev-static-1)</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t>The product upload dialog button is now 파일로 주문하기 and the file-type copy reads 'ai · psd · pdf · eps · tif · png · jpg'. ProductV2Page.expectDesignUploadModal and MS-V2-053 will fail when this reaches production - update storefront-data.ts then.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>MS-V2-058</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="inlineStr">
+        <is>
+          <t>Marked test.fixme (known alt-text defect on the size guide); skipped until fixed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37"/>
+    <row r="38">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-10 - test-case.md v1</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
           <t>Origin</t>
         </is>
       </c>
-      <c r="B34" s="5" t="inlineStr">
+      <c r="B39" s="5" t="inlineStr">
         <is>
           <t>Storefront v2 test case matrix (MS-V2-001 onward) and automation standards, now carried by this workbook and docs/CONVENTIONS.md.</t>
         </is>

</xml_diff>